<commit_message>
feat: v0.7.12 Real prompt_tokens at Decision Points
Switch context pressure detection and compression triggering from
estimate_tokens() heuristic to actual prompt_tokens returned by LLM API.
Uses previous iteration's prompt_tokens (falls back to estimate on first
iteration), with verbose deviation logging when estimate differs >10%.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/test_cases.xlsx
+++ b/tests/test_cases.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E519"/>
+  <dimension ref="A1:E539"/>
   <sheetFormatPr baseColWidth="15" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14436,6 +14436,466 @@
         </is>
       </c>
     </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>决策点真实Token</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>TestContextManagerRealTokens</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>真实token覆盖估算</t>
+        </is>
+      </c>
+      <c r="D520" t="inlineStr">
+        <is>
+          <t>提供last_prompt_tokens时使用真实值而非estimate_tokens</t>
+        </is>
+      </c>
+      <c r="E520" t="inlineStr"/>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>决策点真实Token</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>TestContextManagerRealTokens</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>无真实token回退估算</t>
+        </is>
+      </c>
+      <c r="D521" t="inlineStr">
+        <is>
+          <t>last_prompt_tokens=None时回退到estimate_tokens()</t>
+        </is>
+      </c>
+      <c r="E521" t="inlineStr"/>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>决策点真实Token</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>TestContextManagerRealTokens</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>None与不传参数等价</t>
+        </is>
+      </c>
+      <c r="D522" t="inlineStr">
+        <is>
+          <t>last_prompt_tokens=None与不传参数行为一致</t>
+        </is>
+      </c>
+      <c r="E522" t="inlineStr"/>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>决策点真实Token</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>TestContextManagerRealTokens</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>真实token阻止误压缩</t>
+        </is>
+      </c>
+      <c r="D523" t="inlineStr">
+        <is>
+          <t>估算显示超限但真实token显示安全时不压缩</t>
+        </is>
+      </c>
+      <c r="E523" t="inlineStr"/>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>决策点真实Token</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>TestContextManagerRealTokens</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>verbose输出来源标记</t>
+        </is>
+      </c>
+      <c r="D524" t="inlineStr">
+        <is>
+          <t>verbose模式下输出[real]或[estimated]标记</t>
+        </is>
+      </c>
+      <c r="E524" t="inlineStr"/>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>决策点真实Token</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>TestCompressorRealTokens</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>should_compress使用真实token</t>
+        </is>
+      </c>
+      <c r="D525" t="inlineStr">
+        <is>
+          <t>提供last_prompt_tokens时直接与threshold比较</t>
+        </is>
+      </c>
+      <c r="E525" t="inlineStr"/>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>决策点真实Token</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>TestCompressorRealTokens</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>should_compress回退估算</t>
+        </is>
+      </c>
+      <c r="D526" t="inlineStr">
+        <is>
+          <t>last_prompt_tokens=None时使用estimate_tokens</t>
+        </is>
+      </c>
+      <c r="E526" t="inlineStr"/>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>决策点真实Token</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>TestCompressorRealTokens</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>compress透传last_prompt_tokens</t>
+        </is>
+      </c>
+      <c r="D527" t="inlineStr">
+        <is>
+          <t>compress()将last_prompt_tokens传递给should_compress()</t>
+        </is>
+      </c>
+      <c r="E527" t="inlineStr"/>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>决策点真实Token</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>TestCompressorRealTokens</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>真实token低于阈值不压缩</t>
+        </is>
+      </c>
+      <c r="D528" t="inlineStr">
+        <is>
+          <t>real tokens &lt; threshold时compress返回原消息列表</t>
+        </is>
+      </c>
+      <c r="E528" t="inlineStr"/>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>决策点真实Token</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>TestCompressorRealTokens</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>禁用压缩器忽略真实token</t>
+        </is>
+      </c>
+      <c r="D529" t="inlineStr">
+        <is>
+          <t>enabled=False时无论真实token多高都不压缩</t>
+        </is>
+      </c>
+      <c r="E529" t="inlineStr"/>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>决策点真实Token</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>TestReActAgentRealTokenIntegration</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>初始状态为None</t>
+        </is>
+      </c>
+      <c r="D530" t="inlineStr">
+        <is>
+          <t>_last_prompt_tokens初始化为None</t>
+        </is>
+      </c>
+      <c r="E530" t="inlineStr"/>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>决策点真实Token</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>TestReActAgentRealTokenIntegration</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>LLM调用后存储真实token</t>
+        </is>
+      </c>
+      <c r="D531" t="inlineStr">
+        <is>
+          <t>usage.prompt_tokens&gt;0时更新_last_prompt_tokens</t>
+        </is>
+      </c>
+      <c r="E531" t="inlineStr"/>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>决策点真实Token</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>TestReActAgentRealTokenIntegration</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>_prepare_run重置token</t>
+        </is>
+      </c>
+      <c r="D532" t="inlineStr">
+        <is>
+          <t>_prepare_run()将_last_prompt_tokens重置为None</t>
+        </is>
+      </c>
+      <c r="E532" t="inlineStr"/>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>决策点真实Token</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>TestReActAgentRealTokenIntegration</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>check_and_compress接收真实token</t>
+        </is>
+      </c>
+      <c r="D533" t="inlineStr">
+        <is>
+          <t>_think()传递_last_prompt_tokens给check_and_compress</t>
+        </is>
+      </c>
+      <c r="E533" t="inlineStr"/>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>决策点真实Token</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>TestReActAgentRealTokenIntegration</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>should_compress接收真实token</t>
+        </is>
+      </c>
+      <c r="D534" t="inlineStr">
+        <is>
+          <t>_think()传递_last_prompt_tokens给should_compress</t>
+        </is>
+      </c>
+      <c r="E534" t="inlineStr"/>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>决策点真实Token</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>TestReActAgentRealTokenIntegration</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>compress接收真实token</t>
+        </is>
+      </c>
+      <c r="D535" t="inlineStr">
+        <is>
+          <t>_think()传递_last_prompt_tokens给compress</t>
+        </is>
+      </c>
+      <c r="E535" t="inlineStr"/>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>决策点真实Token</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>TestBackwardCompatibility</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>check_and_compress无需新参数</t>
+        </is>
+      </c>
+      <c r="D536" t="inlineStr">
+        <is>
+          <t>不传last_prompt_tokens时check_and_compress正常工作</t>
+        </is>
+      </c>
+      <c r="E536" t="inlineStr"/>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>决策点真实Token</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>TestBackwardCompatibility</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>should_compress无需新参数</t>
+        </is>
+      </c>
+      <c r="D537" t="inlineStr">
+        <is>
+          <t>不传last_prompt_tokens时should_compress正常工作</t>
+        </is>
+      </c>
+      <c r="E537" t="inlineStr"/>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>决策点真实Token</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>TestBackwardCompatibility</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>compress无需新参数</t>
+        </is>
+      </c>
+      <c r="D538" t="inlineStr">
+        <is>
+          <t>不传last_prompt_tokens时compress正常工作</t>
+        </is>
+      </c>
+      <c r="E538" t="inlineStr"/>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>决策点真实Token</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>TestBackwardCompatibility</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>estimate_tokens仍可用</t>
+        </is>
+      </c>
+      <c r="D539" t="inlineStr">
+        <is>
+          <t>estimate_tokens()作为回退仍可正常调用</t>
+        </is>
+      </c>
+      <c r="E539" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: v0.7.17 多轮缓存与 Tool Offloading
- Tool Offloading: 大结果写入临时文件，仅注入摘要+路径引用到上下文
- 多轮缓存: 跨轮次复用工具结果，支持磁盘持久化与mtime失效
- BaseTool.can_offload 属性，5个内置工具启用
- CacheEntry 数据结构扩展（file_mtimes, is_offloaded）
- 缓存预热/持久化/warmup_on_restore 配置支持
- 修复 PluginsConfig 缺失解析/保存，更新文档与 test_cases.xlsx
- 全量测试 1162 passed

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/test_cases.xlsx
+++ b/tests/test_cases.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E652"/>
+  <dimension ref="A1:E684"/>
   <sheetFormatPr baseColWidth="15" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17387,6 +17387,710 @@
         </is>
       </c>
     </row>
+    <row r="653">
+      <c r="A653" t="inlineStr">
+        <is>
+          <t>Tool Offload</t>
+        </is>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>TestToolOffloadConfig</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>默认配置</t>
+        </is>
+      </c>
+      <c r="D653" t="inlineStr">
+        <is>
+          <t>enabled=True, size_threshold=1000, auto_cleanup=True</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="inlineStr">
+        <is>
+          <t>Tool Offload</t>
+        </is>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>TestToolOffloadConfig</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>自定义配置</t>
+        </is>
+      </c>
+      <c r="D654" t="inlineStr">
+        <is>
+          <t>自定义 enabled/size_threshold/offload_dir</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="inlineStr">
+        <is>
+          <t>Tool Offload</t>
+        </is>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>TestToolOffloadManager</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>禁用时不卸载</t>
+        </is>
+      </c>
+      <c r="D655" t="inlineStr">
+        <is>
+          <t>enabled=False → should_offload=False</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="inlineStr">
+        <is>
+          <t>Tool Offload</t>
+        </is>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>TestToolOffloadManager</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>工具不支持不卸载</t>
+        </is>
+      </c>
+      <c r="D656" t="inlineStr">
+        <is>
+          <t>can_offload=False → should_offload=False</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="inlineStr">
+        <is>
+          <t>Tool Offload</t>
+        </is>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>TestToolOffloadManager</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>低于阈值不卸载</t>
+        </is>
+      </c>
+      <c r="D657" t="inlineStr">
+        <is>
+          <t>小内容 → should_offload=False</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>Tool Offload</t>
+        </is>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>TestToolOffloadManager</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>超过阈值触发卸载</t>
+        </is>
+      </c>
+      <c r="D658" t="inlineStr">
+        <is>
+          <t>大内容+can_offload → should_offload=True</t>
+        </is>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="inlineStr">
+        <is>
+          <t>Tool Offload</t>
+        </is>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>TestToolOffloadManager</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>排除工具不卸载</t>
+        </is>
+      </c>
+      <c r="D659" t="inlineStr">
+        <is>
+          <t>memorize → should_offload=False</t>
+        </is>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="inlineStr">
+        <is>
+          <t>Tool Offload</t>
+        </is>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>TestToolOffloadManager</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>卸载写文件</t>
+        </is>
+      </c>
+      <c r="D660" t="inlineStr">
+        <is>
+          <t>offload() → 临时文件存在且内容正确</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="inlineStr">
+        <is>
+          <t>Tool Offload</t>
+        </is>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>TestToolOffloadManager</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>卸载返回摘要</t>
+        </is>
+      </c>
+      <c r="D661" t="inlineStr">
+        <is>
+          <t>摘要包含 [结果已卸载] 和 file_read 路径</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>Tool Offload</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>TestToolOffloadManager</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>卸载跟踪元数据</t>
+        </is>
+      </c>
+      <c r="D662" t="inlineStr">
+        <is>
+          <t>original_size_tokens &gt; 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>Tool Offload</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>TestToolOffloadManager</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>cleanup清理文件</t>
+        </is>
+      </c>
+      <c r="D663" t="inlineStr">
+        <is>
+          <t>cleanup() → 临时文件删除</t>
+        </is>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>Tool Offload</t>
+        </is>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>TestToolOffloadManager</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>统计信息</t>
+        </is>
+      </c>
+      <c r="D664" t="inlineStr">
+        <is>
+          <t>get_stats() → offloaded_count, total_tokens_saved</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="inlineStr">
+        <is>
+          <t>Tool Offload</t>
+        </is>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>TestToolOffloadManager</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>按ID查询</t>
+        </is>
+      </c>
+      <c r="D665" t="inlineStr">
+        <is>
+          <t>get_offloaded() → 正确结果且 accessed=True</t>
+        </is>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>Tool Offload</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>TestToolOffloadManager</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>按路径查询</t>
+        </is>
+      </c>
+      <c r="D666" t="inlineStr">
+        <is>
+          <t>get_by_path() → 正确结果</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>Tool Offload</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>TestBaseToolCanOffload</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>默认can_offload</t>
+        </is>
+      </c>
+      <c r="D667" t="inlineStr">
+        <is>
+          <t>BaseTool.can_offload=False</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>Tool Offload</t>
+        </is>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>TestBaseToolCanOffload</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>设置can_offload</t>
+        </is>
+      </c>
+      <c r="D668" t="inlineStr">
+        <is>
+          <t>can_offload=True 生效</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>Multi-turn Cache</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>TestCacheConfigExtended</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>默认多轮字段</t>
+        </is>
+      </c>
+      <c r="D669" t="inlineStr">
+        <is>
+          <t>persist=False, warmup_on_restore=True, mtime_invalidation=True</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>Multi-turn Cache</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>TestCacheConfigExtended</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>自定义多轮字段</t>
+        </is>
+      </c>
+      <c r="D670" t="inlineStr">
+        <is>
+          <t>自定义 persist/persist_dir/warmup_on_restore</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>Multi-turn Cache</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>TestCacheMtimeInvalidation</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>mtime变化失效</t>
+        </is>
+      </c>
+      <c r="D671" t="inlineStr">
+        <is>
+          <t>文件修改后缓存失效</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>Multi-turn Cache</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>TestCacheMtimeInvalidation</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>mtime不变有效</t>
+        </is>
+      </c>
+      <c r="D672" t="inlineStr">
+        <is>
+          <t>文件未修改缓存有效</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>Multi-turn Cache</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>TestCacheMtimeInvalidation</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>非文件工具无mtime检查</t>
+        </is>
+      </c>
+      <c r="D673" t="inlineStr">
+        <is>
+          <t>shell_execute 不受 mtime 影响</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>Multi-turn Cache</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>TestCacheMtimeInvalidation</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>自动提取文件路径</t>
+        </is>
+      </c>
+      <c r="D674" t="inlineStr">
+        <is>
+          <t>从 args 自动提取 file_path</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>Multi-turn Cache</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>TestCacheMtimeInvalidation</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>禁用mtime检查</t>
+        </is>
+      </c>
+      <c r="D675" t="inlineStr">
+        <is>
+          <t>mtime_invalidation=False → 文件修改不影响</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>Multi-turn Cache</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>TestCachePersistence</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>持久化到磁盘</t>
+        </is>
+      </c>
+      <c r="D676" t="inlineStr">
+        <is>
+          <t>persist_to_disk() → manifest.json 存在</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>Multi-turn Cache</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>TestCachePersistence</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>从磁盘预热</t>
+        </is>
+      </c>
+      <c r="D677" t="inlineStr">
+        <is>
+          <t>warmup_from_disk() → 加载缓存</t>
+        </is>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>Multi-turn Cache</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>TestCachePersistence</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>跳过过期条目</t>
+        </is>
+      </c>
+      <c r="D678" t="inlineStr">
+        <is>
+          <t>过期条目不加载</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>Multi-turn Cache</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>TestCachePersistence</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>跳过过期文件</t>
+        </is>
+      </c>
+      <c r="D679" t="inlineStr">
+        <is>
+          <t>mtime 变化的条目不加载</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>Multi-turn Cache</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>TestCachePersistence</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>空manifest</t>
+        </is>
+      </c>
+      <c r="D680" t="inlineStr">
+        <is>
+          <t>不存在的目录 → 返回 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>Multi-turn Cache</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>TestCacheOffloadIntegration</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>缓存存储卸载摘要</t>
+        </is>
+      </c>
+      <c r="D681" t="inlineStr">
+        <is>
+          <t>is_offloaded=True 时缓存摘要</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>Multi-turn Cache</t>
+        </is>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>TestCacheOffloadIntegration</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>统计跟踪卸载条目</t>
+        </is>
+      </c>
+      <c r="D682" t="inlineStr">
+        <is>
+          <t>offloaded_entries 计数正确</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>Multi-turn Cache</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>TestCacheEntry</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>offload标志</t>
+        </is>
+      </c>
+      <c r="D683" t="inlineStr">
+        <is>
+          <t>is_offloaded=True</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>Multi-turn Cache</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>TestCacheEntry</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>文件mtime</t>
+        </is>
+      </c>
+      <c r="D684" t="inlineStr">
+        <is>
+          <t>file_mtimes 正确记录</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: 更新 test_cases.xlsx + 改进 check_test_cases.sh 检测已有文件新增方法
新增 6 个 base_ratio 首轮偏差修正测试用例到 xlsx。
改进 pre-commit hook：除了检测新增文件，也检测已有测试文件的新增类/方法。

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/test_cases.xlsx
+++ b/tests/test_cases.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E722"/>
+  <dimension ref="A1:E728"/>
   <sheetFormatPr baseColWidth="15" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18927,6 +18927,138 @@
         </is>
       </c>
     </row>
+    <row r="723">
+      <c r="A723" t="inlineStr">
+        <is>
+          <t>Estimation Audit</t>
+        </is>
+      </c>
+      <c r="B723" t="inlineStr">
+        <is>
+          <t>TestBaseRatioFirstRoundCorrection</t>
+        </is>
+      </c>
+      <c r="C723" t="inlineStr">
+        <is>
+          <t>单轮迭代不设 base_ratio</t>
+        </is>
+      </c>
+      <c r="D723" t="inlineStr">
+        <is>
+          <t>单轮迭代 run 不设置 base_ratio，使用 per-iteration ratio</t>
+        </is>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" t="inlineStr">
+        <is>
+          <t>Estimation Audit</t>
+        </is>
+      </c>
+      <c r="B724" t="inlineStr">
+        <is>
+          <t>TestBaseRatioFirstRoundCorrection</t>
+        </is>
+      </c>
+      <c r="C724" t="inlineStr">
+        <is>
+          <t>两轮迭代从第二轮设 base_ratio</t>
+        </is>
+      </c>
+      <c r="D724" t="inlineStr">
+        <is>
+          <t>两轮迭代 run 从第二轮设置 base_ratio</t>
+        </is>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" t="inlineStr">
+        <is>
+          <t>Estimation Audit</t>
+        </is>
+      </c>
+      <c r="B725" t="inlineStr">
+        <is>
+          <t>TestBaseRatioFirstRoundCorrection</t>
+        </is>
+      </c>
+      <c r="C725" t="inlineStr">
+        <is>
+          <t>三轮迭代 base_ratio 稳定</t>
+        </is>
+      </c>
+      <c r="D725" t="inlineStr">
+        <is>
+          <t>三轮迭代 base_ratio 从第二轮设置，第三轮保持一致</t>
+        </is>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" t="inlineStr">
+        <is>
+          <t>Estimation Audit</t>
+        </is>
+      </c>
+      <c r="B726" t="inlineStr">
+        <is>
+          <t>TestBaseRatioFirstRoundCorrection</t>
+        </is>
+      </c>
+      <c r="C726" t="inlineStr">
+        <is>
+          <t>跨 run 重置 base_ratio</t>
+        </is>
+      </c>
+      <c r="D726" t="inlineStr">
+        <is>
+          <t>start_run() 重置 base_ratio 相关字段</t>
+        </is>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" t="inlineStr">
+        <is>
+          <t>Estimation Audit</t>
+        </is>
+      </c>
+      <c r="B727" t="inlineStr">
+        <is>
+          <t>TestBaseRatioFirstRoundCorrection</t>
+        </is>
+      </c>
+      <c r="C727" t="inlineStr">
+        <is>
+          <t>首轮 breakdown 准确</t>
+        </is>
+      </c>
+      <c r="D727" t="inlineStr">
+        <is>
+          <t>首轮使用 per-iteration ratio，token 分类之和等于 prompt_tokens</t>
+        </is>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" t="inlineStr">
+        <is>
+          <t>Estimation Audit</t>
+        </is>
+      </c>
+      <c r="B728" t="inlineStr">
+        <is>
+          <t>TestBaseRatioFirstRoundCorrection</t>
+        </is>
+      </c>
+      <c r="C728" t="inlineStr">
+        <is>
+          <t>message_tokens 不为负</t>
+        </is>
+      </c>
+      <c r="D728" t="inlineStr">
+        <is>
+          <t>max(0,...) 守卫确保 message_tokens &gt;= 0</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: v0.8.3 输入净化 — Prompt injection 硬拦截 + 格式/长度校验
在 orchestrator 入口加一道安检，用户输入经三步净化后才进入 ReAct 循环：
1. 格式检查 — null bytes 拒绝 + 控制字符剥离（str.maketrans 高效实现）
2. 注入检查 — 18 个中英文注入模式正则匹配，命中硬拒绝
3. 长度检查 — 整体截断/拒绝 + 单行截断

核心变更：
- 新增 InputSanitizer + SanitizerResult (sanitizer.py)
- SanitizerConfig 8 个配置字段 + 18 个默认注入模式 (schema.py)
- AgentOrchestrator.run() sanitizer 门控，拒绝返回 INPUT_REJECTED
- AgentBuilder 配置接线，CLI 交互循环拒绝处理 + /config 显示
- TerminationReason/AgentEvent 新增 INPUT_REJECTED 枚举
- 47 个单元测试：配置/格式/注入/长度/集成/边界

/simplify 修复：
- 提取 _reject() 辅助方法消除 3 处重复拒绝路径
- str.maketrans 替代 O(n) Python 循环剥离控制字符
- 移除 orchestrator 重复 INPUT_REJECTED 事件发射
- CLI 使用 TerminationReason.INPUT_REJECTED.value 替代硬编码字符串

文档更新：
- docs/api.md: SanitizerConfig + InputSanitizer API 文档
- docs/constraints.md: 输入净化约束 + 交互流程图
- docs/architecture.md: 净化门控节点 + 数据流
- docs/tutorial.md: 配置示例 + 安全 FAQ

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/test_cases.xlsx
+++ b/tests/test_cases.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E855"/>
+  <dimension ref="A1:E902"/>
   <sheetFormatPr baseColWidth="15" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21126,7 +21126,6 @@
           <t>新限流器初始令牌数等于 burst</t>
         </is>
       </c>
-      <c r="E822" t="inlineStr"/>
     </row>
     <row r="823">
       <c r="A823" t="inlineStr">
@@ -21149,7 +21148,6 @@
           <t>acquire() 扣减 1 个令牌</t>
         </is>
       </c>
-      <c r="E823" t="inlineStr"/>
     </row>
     <row r="824">
       <c r="A824" t="inlineStr">
@@ -21172,7 +21170,6 @@
           <t>令牌按时间速率恢复</t>
         </is>
       </c>
-      <c r="E824" t="inlineStr"/>
     </row>
     <row r="825">
       <c r="A825" t="inlineStr">
@@ -21195,7 +21192,6 @@
           <t>令牌为 0 时 acquire 阻塞并返回等待时间</t>
         </is>
       </c>
-      <c r="E825" t="inlineStr"/>
     </row>
     <row r="826">
       <c r="A826" t="inlineStr">
@@ -21218,7 +21214,6 @@
           <t>允许 burst 次突发请求</t>
         </is>
       </c>
-      <c r="E826" t="inlineStr"/>
     </row>
     <row r="827">
       <c r="A827" t="inlineStr">
@@ -21241,7 +21236,6 @@
           <t>令牌数不超过 max_tokens</t>
         </is>
       </c>
-      <c r="E827" t="inlineStr"/>
     </row>
     <row r="828">
       <c r="A828" t="inlineStr">
@@ -21264,7 +21258,6 @@
           <t>reset() 恢复满桶</t>
         </is>
       </c>
-      <c r="E828" t="inlineStr"/>
     </row>
     <row r="829">
       <c r="A829" t="inlineStr">
@@ -21287,7 +21280,6 @@
           <t>有令牌时立即执行</t>
         </is>
       </c>
-      <c r="E829" t="inlineStr"/>
     </row>
     <row r="830">
       <c r="A830" t="inlineStr">
@@ -21310,7 +21302,6 @@
           <t>限流等待时触发 on_wait 回调</t>
         </is>
       </c>
-      <c r="E830" t="inlineStr"/>
     </row>
     <row r="831">
       <c r="A831" t="inlineStr">
@@ -21333,7 +21324,6 @@
           <t>无限流时不触发回调</t>
         </is>
       </c>
-      <c r="E831" t="inlineStr"/>
     </row>
     <row r="832">
       <c r="A832" t="inlineStr">
@@ -21356,7 +21346,6 @@
           <t>返回值透传</t>
         </is>
       </c>
-      <c r="E832" t="inlineStr"/>
     </row>
     <row r="833">
       <c r="A833" t="inlineStr">
@@ -21379,7 +21368,6 @@
           <t>默认配置值正确</t>
         </is>
       </c>
-      <c r="E833" t="inlineStr"/>
     </row>
     <row r="834">
       <c r="A834" t="inlineStr">
@@ -21402,7 +21390,6 @@
           <t>Config.rate_limiter 存在且类型正确</t>
         </is>
       </c>
-      <c r="E834" t="inlineStr"/>
     </row>
     <row r="835">
       <c r="A835" t="inlineStr">
@@ -21425,7 +21412,6 @@
           <t>_from_dict 解析 rate_limiter 配置</t>
         </is>
       </c>
-      <c r="E835" t="inlineStr"/>
     </row>
     <row r="836">
       <c r="A836" t="inlineStr">
@@ -21448,7 +21434,6 @@
           <t>YAML 往返序列化</t>
         </is>
       </c>
-      <c r="E836" t="inlineStr"/>
     </row>
     <row r="837">
       <c r="A837" t="inlineStr">
@@ -21471,7 +21456,6 @@
           <t>enabled 时 chat() 走限流路径</t>
         </is>
       </c>
-      <c r="E837" t="inlineStr"/>
     </row>
     <row r="838">
       <c r="A838" t="inlineStr">
@@ -21494,7 +21478,6 @@
           <t>disabled 时跳过限流</t>
         </is>
       </c>
-      <c r="E838" t="inlineStr"/>
     </row>
     <row r="839">
       <c r="A839" t="inlineStr">
@@ -21517,7 +21500,6 @@
           <t>config 为 None 时跳过限流</t>
         </is>
       </c>
-      <c r="E839" t="inlineStr"/>
     </row>
     <row r="840">
       <c r="A840" t="inlineStr">
@@ -21540,7 +21522,6 @@
           <t>限流器包裹重试，两层同时生效</t>
         </is>
       </c>
-      <c r="E840" t="inlineStr"/>
     </row>
     <row r="841">
       <c r="A841" t="inlineStr">
@@ -21563,7 +21544,6 @@
           <t>限流时 _on_rate_limit_callback 被调用</t>
         </is>
       </c>
-      <c r="E841" t="inlineStr"/>
     </row>
     <row r="842">
       <c r="A842" t="inlineStr">
@@ -21586,7 +21566,6 @@
           <t>requests_per_minute=0 抛 ValueError</t>
         </is>
       </c>
-      <c r="E842" t="inlineStr"/>
     </row>
     <row r="843">
       <c r="A843" t="inlineStr">
@@ -21609,7 +21588,6 @@
           <t>requests_per_minute&lt;0 抛 ValueError</t>
         </is>
       </c>
-      <c r="E843" t="inlineStr"/>
     </row>
     <row r="844">
       <c r="A844" t="inlineStr">
@@ -21632,7 +21610,6 @@
           <t>burst=0 抛 ValueError</t>
         </is>
       </c>
-      <c r="E844" t="inlineStr"/>
     </row>
     <row r="845">
       <c r="A845" t="inlineStr">
@@ -21655,7 +21632,6 @@
           <t>burst&lt;0 抛 ValueError</t>
         </is>
       </c>
-      <c r="E845" t="inlineStr"/>
     </row>
     <row r="846">
       <c r="A846" t="inlineStr">
@@ -21678,7 +21654,6 @@
           <t>合法配置不抛异常</t>
         </is>
       </c>
-      <c r="E846" t="inlineStr"/>
     </row>
     <row r="847">
       <c r="A847" t="inlineStr">
@@ -21701,7 +21676,6 @@
           <t>Builder 注入 rate_limiter_config 和 limiter 实例</t>
         </is>
       </c>
-      <c r="E847" t="inlineStr"/>
     </row>
     <row r="848">
       <c r="A848" t="inlineStr">
@@ -21724,7 +21698,6 @@
           <t>enabled 时连接回调</t>
         </is>
       </c>
-      <c r="E848" t="inlineStr"/>
     </row>
     <row r="849">
       <c r="A849" t="inlineStr">
@@ -21747,7 +21720,6 @@
           <t>disabled 时不连接回调</t>
         </is>
       </c>
-      <c r="E849" t="inlineStr"/>
     </row>
     <row r="850">
       <c r="A850" t="inlineStr">
@@ -21770,7 +21742,6 @@
           <t>限流时发射 LLM_RATE_LIMITED 事件</t>
         </is>
       </c>
-      <c r="E850" t="inlineStr"/>
     </row>
     <row r="851">
       <c r="A851" t="inlineStr">
@@ -21793,7 +21764,6 @@
           <t>限流器+重试两层同时活跃</t>
         </is>
       </c>
-      <c r="E851" t="inlineStr"/>
     </row>
     <row r="852">
       <c r="A852" t="inlineStr">
@@ -21816,7 +21786,6 @@
           <t>disabled 时 _apply_rate_limit 无操作</t>
         </is>
       </c>
-      <c r="E852" t="inlineStr"/>
     </row>
     <row r="853">
       <c r="A853" t="inlineStr">
@@ -21839,7 +21808,6 @@
           <t>config 为 None 时无操作</t>
         </is>
       </c>
-      <c r="E853" t="inlineStr"/>
     </row>
     <row r="854">
       <c r="A854" t="inlineStr">
@@ -21862,7 +21830,6 @@
           <t>enabled 时获取令牌</t>
         </is>
       </c>
-      <c r="E854" t="inlineStr"/>
     </row>
     <row r="855">
       <c r="A855" t="inlineStr">
@@ -21885,7 +21852,1040 @@
           <t>限流时触发回调</t>
         </is>
       </c>
-      <c r="E855" t="inlineStr"/>
+    </row>
+    <row r="856">
+      <c r="A856" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B856" t="inlineStr">
+        <is>
+          <t>TestSanitizerConfig</t>
+        </is>
+      </c>
+      <c r="C856" t="inlineStr">
+        <is>
+          <t>default_config</t>
+        </is>
+      </c>
+      <c r="D856" t="inlineStr">
+        <is>
+          <t>默认配置值正确</t>
+        </is>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B857" t="inlineStr">
+        <is>
+          <t>TestSanitizerConfig</t>
+        </is>
+      </c>
+      <c r="C857" t="inlineStr">
+        <is>
+          <t>custom_config</t>
+        </is>
+      </c>
+      <c r="D857" t="inlineStr">
+        <is>
+          <t>自定义配置生效</t>
+        </is>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B858" t="inlineStr">
+        <is>
+          <t>TestSanitizerConfig</t>
+        </is>
+      </c>
+      <c r="C858" t="inlineStr">
+        <is>
+          <t>config_in_full_config</t>
+        </is>
+      </c>
+      <c r="D858" t="inlineStr">
+        <is>
+          <t>Config 中包含 sanitizer 字段</t>
+        </is>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B859" t="inlineStr">
+        <is>
+          <t>TestSanitizerConfig</t>
+        </is>
+      </c>
+      <c r="C859" t="inlineStr">
+        <is>
+          <t>custom_patterns_appended</t>
+        </is>
+      </c>
+      <c r="D859" t="inlineStr">
+        <is>
+          <t>自定义模式追加到默认列表</t>
+        </is>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B860" t="inlineStr">
+        <is>
+          <t>TestSanitizerConfig</t>
+        </is>
+      </c>
+      <c r="C860" t="inlineStr">
+        <is>
+          <t>config_from_dict</t>
+        </is>
+      </c>
+      <c r="D860" t="inlineStr">
+        <is>
+          <t>_from_dict 反序列化正确</t>
+        </is>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B861" t="inlineStr">
+        <is>
+          <t>TestSanitizerConfig</t>
+        </is>
+      </c>
+      <c r="C861" t="inlineStr">
+        <is>
+          <t>injection_patterns_default_count</t>
+        </is>
+      </c>
+      <c r="D861" t="inlineStr">
+        <is>
+          <t>默认注入模式数量为 18</t>
+        </is>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B862" t="inlineStr">
+        <is>
+          <t>TestSanitizerResult</t>
+        </is>
+      </c>
+      <c r="C862" t="inlineStr">
+        <is>
+          <t>result_fields</t>
+        </is>
+      </c>
+      <c r="D862" t="inlineStr">
+        <is>
+          <t>SanitizerResult 字段正确</t>
+        </is>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B863" t="inlineStr">
+        <is>
+          <t>TestSanitizerResult</t>
+        </is>
+      </c>
+      <c r="C863" t="inlineStr">
+        <is>
+          <t>result_rejected</t>
+        </is>
+      </c>
+      <c r="D863" t="inlineStr">
+        <is>
+          <t>被拒绝结果字段正确</t>
+        </is>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B864" t="inlineStr">
+        <is>
+          <t>TestSanitizerResult</t>
+        </is>
+      </c>
+      <c r="C864" t="inlineStr">
+        <is>
+          <t>result_with_actions</t>
+        </is>
+      </c>
+      <c r="D864" t="inlineStr">
+        <is>
+          <t>带 actions 的结果正确</t>
+        </is>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B865" t="inlineStr">
+        <is>
+          <t>TestFormatValidation</t>
+        </is>
+      </c>
+      <c r="C865" t="inlineStr">
+        <is>
+          <t>clean_input_passes</t>
+        </is>
+      </c>
+      <c r="D865" t="inlineStr">
+        <is>
+          <t>干净输入通过</t>
+        </is>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B866" t="inlineStr">
+        <is>
+          <t>TestFormatValidation</t>
+        </is>
+      </c>
+      <c r="C866" t="inlineStr">
+        <is>
+          <t>null_bytes_rejected</t>
+        </is>
+      </c>
+      <c r="D866" t="inlineStr">
+        <is>
+          <t>null bytes 被拒绝</t>
+        </is>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B867" t="inlineStr">
+        <is>
+          <t>TestFormatValidation</t>
+        </is>
+      </c>
+      <c r="C867" t="inlineStr">
+        <is>
+          <t>null_bytes_disabled</t>
+        </is>
+      </c>
+      <c r="D867" t="inlineStr">
+        <is>
+          <t>禁用时不拒绝 null bytes</t>
+        </is>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B868" t="inlineStr">
+        <is>
+          <t>TestFormatValidation</t>
+        </is>
+      </c>
+      <c r="C868" t="inlineStr">
+        <is>
+          <t>control_chars_stripped</t>
+        </is>
+      </c>
+      <c r="D868" t="inlineStr">
+        <is>
+          <t>控制字符被剥离</t>
+        </is>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B869" t="inlineStr">
+        <is>
+          <t>TestFormatValidation</t>
+        </is>
+      </c>
+      <c r="C869" t="inlineStr">
+        <is>
+          <t>tab_newline_preserved</t>
+        </is>
+      </c>
+      <c r="D869" t="inlineStr">
+        <is>
+          <t>tab/newline/CR 保留</t>
+        </is>
+      </c>
+    </row>
+    <row r="870">
+      <c r="A870" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B870" t="inlineStr">
+        <is>
+          <t>TestFormatValidation</t>
+        </is>
+      </c>
+      <c r="C870" t="inlineStr">
+        <is>
+          <t>ansi_escape_stripped</t>
+        </is>
+      </c>
+      <c r="D870" t="inlineStr">
+        <is>
+          <t>ANSI escape 被剥离</t>
+        </is>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B871" t="inlineStr">
+        <is>
+          <t>TestFormatValidation</t>
+        </is>
+      </c>
+      <c r="C871" t="inlineStr">
+        <is>
+          <t>mixed_control_chars</t>
+        </is>
+      </c>
+      <c r="D871" t="inlineStr">
+        <is>
+          <t>混合控制字符处理正确</t>
+        </is>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B872" t="inlineStr">
+        <is>
+          <t>TestInjectionPatterns</t>
+        </is>
+      </c>
+      <c r="C872" t="inlineStr">
+        <is>
+          <t>ignore_previous_instructions_rejected</t>
+        </is>
+      </c>
+      <c r="D872" t="inlineStr">
+        <is>
+          <t>"ignore previous instructions" 被拒绝</t>
+        </is>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B873" t="inlineStr">
+        <is>
+          <t>TestInjectionPatterns</t>
+        </is>
+      </c>
+      <c r="C873" t="inlineStr">
+        <is>
+          <t>disregard_all_rules_rejected</t>
+        </is>
+      </c>
+      <c r="D873" t="inlineStr">
+        <is>
+          <t>"disregard all rules" 被拒绝</t>
+        </is>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B874" t="inlineStr">
+        <is>
+          <t>TestInjectionPatterns</t>
+        </is>
+      </c>
+      <c r="C874" t="inlineStr">
+        <is>
+          <t>you_are_now_rejected</t>
+        </is>
+      </c>
+      <c r="D874" t="inlineStr">
+        <is>
+          <t>"You are now" 被拒绝</t>
+        </is>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B875" t="inlineStr">
+        <is>
+          <t>TestInjectionPatterns</t>
+        </is>
+      </c>
+      <c r="C875" t="inlineStr">
+        <is>
+          <t>dan_jailbreak_rejected</t>
+        </is>
+      </c>
+      <c r="D875" t="inlineStr">
+        <is>
+          <t>DAN/jailbreak 模式被拒绝</t>
+        </is>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B876" t="inlineStr">
+        <is>
+          <t>TestInjectionPatterns</t>
+        </is>
+      </c>
+      <c r="C876" t="inlineStr">
+        <is>
+          <t>chinese_ignore_instructions_rejected</t>
+        </is>
+      </c>
+      <c r="D876" t="inlineStr">
+        <is>
+          <t>中文"忽略之前的指令"被拒绝</t>
+        </is>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B877" t="inlineStr">
+        <is>
+          <t>TestInjectionPatterns</t>
+        </is>
+      </c>
+      <c r="C877" t="inlineStr">
+        <is>
+          <t>chinese_role_hijack_rejected</t>
+        </is>
+      </c>
+      <c r="D877" t="inlineStr">
+        <is>
+          <t>中文"你现在是"被拒绝</t>
+        </is>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B878" t="inlineStr">
+        <is>
+          <t>TestInjectionPatterns</t>
+        </is>
+      </c>
+      <c r="C878" t="inlineStr">
+        <is>
+          <t>case_insensitive_match</t>
+        </is>
+      </c>
+      <c r="D878" t="inlineStr">
+        <is>
+          <t>大小写不敏感匹配</t>
+        </is>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B879" t="inlineStr">
+        <is>
+          <t>TestInjectionPatterns</t>
+        </is>
+      </c>
+      <c r="C879" t="inlineStr">
+        <is>
+          <t>injection_embedded_in_longer_text</t>
+        </is>
+      </c>
+      <c r="D879" t="inlineStr">
+        <is>
+          <t>注入嵌入长文本仍被检测</t>
+        </is>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B880" t="inlineStr">
+        <is>
+          <t>TestInjectionPatterns</t>
+        </is>
+      </c>
+      <c r="C880" t="inlineStr">
+        <is>
+          <t>normal_input_not_rejected</t>
+        </is>
+      </c>
+      <c r="D880" t="inlineStr">
+        <is>
+          <t>正常输入不被误判</t>
+        </is>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B881" t="inlineStr">
+        <is>
+          <t>TestInjectionPatterns</t>
+        </is>
+      </c>
+      <c r="C881" t="inlineStr">
+        <is>
+          <t>custom_pattern_rejected</t>
+        </is>
+      </c>
+      <c r="D881" t="inlineStr">
+        <is>
+          <t>自定义模式生效</t>
+        </is>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B882" t="inlineStr">
+        <is>
+          <t>TestInjectionPatterns</t>
+        </is>
+      </c>
+      <c r="C882" t="inlineStr">
+        <is>
+          <t>injection_disabled_all_passes</t>
+        </is>
+      </c>
+      <c r="D882" t="inlineStr">
+        <is>
+          <t>enabled 是 orchestrator 层守卫</t>
+        </is>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B883" t="inlineStr">
+        <is>
+          <t>TestLengthValidation</t>
+        </is>
+      </c>
+      <c r="C883" t="inlineStr">
+        <is>
+          <t>short_input_passes</t>
+        </is>
+      </c>
+      <c r="D883" t="inlineStr">
+        <is>
+          <t>短输入通过</t>
+        </is>
+      </c>
+    </row>
+    <row r="884">
+      <c r="A884" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B884" t="inlineStr">
+        <is>
+          <t>TestLengthValidation</t>
+        </is>
+      </c>
+      <c r="C884" t="inlineStr">
+        <is>
+          <t>exact_max_length_passes</t>
+        </is>
+      </c>
+      <c r="D884" t="inlineStr">
+        <is>
+          <t>恰好最大长度通过</t>
+        </is>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B885" t="inlineStr">
+        <is>
+          <t>TestLengthValidation</t>
+        </is>
+      </c>
+      <c r="C885" t="inlineStr">
+        <is>
+          <t>over_max_length_truncated</t>
+        </is>
+      </c>
+      <c r="D885" t="inlineStr">
+        <is>
+          <t>超长输入被截断</t>
+        </is>
+      </c>
+    </row>
+    <row r="886">
+      <c r="A886" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B886" t="inlineStr">
+        <is>
+          <t>TestLengthValidation</t>
+        </is>
+      </c>
+      <c r="C886" t="inlineStr">
+        <is>
+          <t>over_max_length_rejected</t>
+        </is>
+      </c>
+      <c r="D886" t="inlineStr">
+        <is>
+          <t>超长输入被拒绝(reject模式)</t>
+        </is>
+      </c>
+    </row>
+    <row r="887">
+      <c r="A887" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B887" t="inlineStr">
+        <is>
+          <t>TestLengthValidation</t>
+        </is>
+      </c>
+      <c r="C887" t="inlineStr">
+        <is>
+          <t>long_line_truncated</t>
+        </is>
+      </c>
+      <c r="D887" t="inlineStr">
+        <is>
+          <t>单行超长被截断</t>
+        </is>
+      </c>
+    </row>
+    <row r="888">
+      <c r="A888" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B888" t="inlineStr">
+        <is>
+          <t>TestLengthValidation</t>
+        </is>
+      </c>
+      <c r="C888" t="inlineStr">
+        <is>
+          <t>max_line_length_zero_unlimited</t>
+        </is>
+      </c>
+      <c r="D888" t="inlineStr">
+        <is>
+          <t>max_line_length=0 不限行长</t>
+        </is>
+      </c>
+    </row>
+    <row r="889">
+      <c r="A889" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B889" t="inlineStr">
+        <is>
+          <t>TestLengthValidation</t>
+        </is>
+      </c>
+      <c r="C889" t="inlineStr">
+        <is>
+          <t>truncation_preserves_valid_utf8</t>
+        </is>
+      </c>
+      <c r="D889" t="inlineStr">
+        <is>
+          <t>截断保留有效 UTF-8</t>
+        </is>
+      </c>
+    </row>
+    <row r="890">
+      <c r="A890" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B890" t="inlineStr">
+        <is>
+          <t>TestSanitizerIntegration</t>
+        </is>
+      </c>
+      <c r="C890" t="inlineStr">
+        <is>
+          <t>orchestrator_rejects_injection</t>
+        </is>
+      </c>
+      <c r="D890" t="inlineStr">
+        <is>
+          <t>orchestrator 拒绝注入输入</t>
+        </is>
+      </c>
+    </row>
+    <row r="891">
+      <c r="A891" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B891" t="inlineStr">
+        <is>
+          <t>TestSanitizerIntegration</t>
+        </is>
+      </c>
+      <c r="C891" t="inlineStr">
+        <is>
+          <t>orchestrator_passes_clean_input</t>
+        </is>
+      </c>
+      <c r="D891" t="inlineStr">
+        <is>
+          <t>orchestrator 放行干净输入</t>
+        </is>
+      </c>
+    </row>
+    <row r="892">
+      <c r="A892" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B892" t="inlineStr">
+        <is>
+          <t>TestSanitizerIntegration</t>
+        </is>
+      </c>
+      <c r="C892" t="inlineStr">
+        <is>
+          <t>sanitizer_disabled_in_orchestrator</t>
+        </is>
+      </c>
+      <c r="D892" t="inlineStr">
+        <is>
+          <t>disabled 时 orchestrator 不拦截</t>
+        </is>
+      </c>
+    </row>
+    <row r="893">
+      <c r="A893" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B893" t="inlineStr">
+        <is>
+          <t>TestSanitizerIntegration</t>
+        </is>
+      </c>
+      <c r="C893" t="inlineStr">
+        <is>
+          <t>sanitizer_event_emitted</t>
+        </is>
+      </c>
+      <c r="D893" t="inlineStr">
+        <is>
+          <t>拒绝时发射 INPUT_REJECTED 事件</t>
+        </is>
+      </c>
+    </row>
+    <row r="894">
+      <c r="A894" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B894" t="inlineStr">
+        <is>
+          <t>TestSanitizerIntegration</t>
+        </is>
+      </c>
+      <c r="C894" t="inlineStr">
+        <is>
+          <t>no_event_on_clean_input</t>
+        </is>
+      </c>
+      <c r="D894" t="inlineStr">
+        <is>
+          <t>干净输入不发射事件</t>
+        </is>
+      </c>
+    </row>
+    <row r="895">
+      <c r="A895" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B895" t="inlineStr">
+        <is>
+          <t>TestSanitizerIntegration</t>
+        </is>
+      </c>
+      <c r="C895" t="inlineStr">
+        <is>
+          <t>execution_result_on_rejection</t>
+        </is>
+      </c>
+      <c r="D895" t="inlineStr">
+        <is>
+          <t>拒绝时返回正确 ExecutionResult</t>
+        </is>
+      </c>
+    </row>
+    <row r="896">
+      <c r="A896" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B896" t="inlineStr">
+        <is>
+          <t>TestSanitizerIntegration</t>
+        </is>
+      </c>
+      <c r="C896" t="inlineStr">
+        <is>
+          <t>orchestrator_truncates_long_input</t>
+        </is>
+      </c>
+      <c r="D896" t="inlineStr">
+        <is>
+          <t>orchestrator 截断超长输入</t>
+        </is>
+      </c>
+    </row>
+    <row r="897">
+      <c r="A897" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B897" t="inlineStr">
+        <is>
+          <t>TestEdgeCases</t>
+        </is>
+      </c>
+      <c r="C897" t="inlineStr">
+        <is>
+          <t>empty_input_passes</t>
+        </is>
+      </c>
+      <c r="D897" t="inlineStr">
+        <is>
+          <t>空输入通过</t>
+        </is>
+      </c>
+    </row>
+    <row r="898">
+      <c r="A898" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B898" t="inlineStr">
+        <is>
+          <t>TestEdgeCases</t>
+        </is>
+      </c>
+      <c r="C898" t="inlineStr">
+        <is>
+          <t>whitespace_only_input_passes</t>
+        </is>
+      </c>
+      <c r="D898" t="inlineStr">
+        <is>
+          <t>纯空白输入通过</t>
+        </is>
+      </c>
+    </row>
+    <row r="899">
+      <c r="A899" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B899" t="inlineStr">
+        <is>
+          <t>TestEdgeCases</t>
+        </is>
+      </c>
+      <c r="C899" t="inlineStr">
+        <is>
+          <t>unicode_input_passes</t>
+        </is>
+      </c>
+      <c r="D899" t="inlineStr">
+        <is>
+          <t>unicode 输入通过</t>
+        </is>
+      </c>
+    </row>
+    <row r="900">
+      <c r="A900" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B900" t="inlineStr">
+        <is>
+          <t>TestEdgeCases</t>
+        </is>
+      </c>
+      <c r="C900" t="inlineStr">
+        <is>
+          <t>code_input_not_flagged</t>
+        </is>
+      </c>
+      <c r="D900" t="inlineStr">
+        <is>
+          <t>代码输入不被误判</t>
+        </is>
+      </c>
+    </row>
+    <row r="901">
+      <c r="A901" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B901" t="inlineStr">
+        <is>
+          <t>TestEdgeCases</t>
+        </is>
+      </c>
+      <c r="C901" t="inlineStr">
+        <is>
+          <t>multiple_violations_first_wins</t>
+        </is>
+      </c>
+      <c r="D901" t="inlineStr">
+        <is>
+          <t>多违规时第一个检查先拦截</t>
+        </is>
+      </c>
+    </row>
+    <row r="902">
+      <c r="A902" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B902" t="inlineStr">
+        <is>
+          <t>TestEdgeCases</t>
+        </is>
+      </c>
+      <c r="C902" t="inlineStr">
+        <is>
+          <t>injection_after_truncation</t>
+        </is>
+      </c>
+      <c r="D902" t="inlineStr">
+        <is>
+          <t>注入在长度检查之前被拦截</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: v0.8.4 PII 脱敏 — phone/id_card/email/api_key 检测 + partial/full 遮蔽 + 重叠处理
Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/test_cases.xlsx
+++ b/tests/test_cases.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E902"/>
+  <dimension ref="A1:E934"/>
   <sheetFormatPr baseColWidth="15" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22887,6 +22887,710 @@
         </is>
       </c>
     </row>
+    <row r="903">
+      <c r="A903" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B903" t="inlineStr">
+        <is>
+          <t>TestPIIDesensitizerPhone</t>
+        </is>
+      </c>
+      <c r="C903" t="inlineStr">
+        <is>
+          <t>chinese_phone_partial_mask</t>
+        </is>
+      </c>
+      <c r="D903" t="inlineStr">
+        <is>
+          <t>中国手机号 partial 遮蔽</t>
+        </is>
+      </c>
+    </row>
+    <row r="904">
+      <c r="A904" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B904" t="inlineStr">
+        <is>
+          <t>TestPIIDesensitizerPhone</t>
+        </is>
+      </c>
+      <c r="C904" t="inlineStr">
+        <is>
+          <t>chinese_phone_full_mask</t>
+        </is>
+      </c>
+      <c r="D904" t="inlineStr">
+        <is>
+          <t>中国手机号 full 遮蔽</t>
+        </is>
+      </c>
+    </row>
+    <row r="905">
+      <c r="A905" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B905" t="inlineStr">
+        <is>
+          <t>TestPIIDesensitizerPhone</t>
+        </is>
+      </c>
+      <c r="C905" t="inlineStr">
+        <is>
+          <t>multiple_phones</t>
+        </is>
+      </c>
+      <c r="D905" t="inlineStr">
+        <is>
+          <t>多个手机号同时遮蔽</t>
+        </is>
+      </c>
+    </row>
+    <row r="906">
+      <c r="A906" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B906" t="inlineStr">
+        <is>
+          <t>TestPIIDesensitizerPhone</t>
+        </is>
+      </c>
+      <c r="C906" t="inlineStr">
+        <is>
+          <t>phone_not_in_text</t>
+        </is>
+      </c>
+      <c r="D906" t="inlineStr">
+        <is>
+          <t>无手机号时不遮蔽</t>
+        </is>
+      </c>
+    </row>
+    <row r="907">
+      <c r="A907" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B907" t="inlineStr">
+        <is>
+          <t>TestPIIDesensitizerIDCard</t>
+        </is>
+      </c>
+      <c r="C907" t="inlineStr">
+        <is>
+          <t>chinese_id_card_partial_mask</t>
+        </is>
+      </c>
+      <c r="D907" t="inlineStr">
+        <is>
+          <t>中国身份证 partial 遮蔽</t>
+        </is>
+      </c>
+    </row>
+    <row r="908">
+      <c r="A908" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B908" t="inlineStr">
+        <is>
+          <t>TestPIIDesensitizerIDCard</t>
+        </is>
+      </c>
+      <c r="C908" t="inlineStr">
+        <is>
+          <t>id_card_with_x</t>
+        </is>
+      </c>
+      <c r="D908" t="inlineStr">
+        <is>
+          <t>身份证末位 X 处理</t>
+        </is>
+      </c>
+    </row>
+    <row r="909">
+      <c r="A909" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B909" t="inlineStr">
+        <is>
+          <t>TestPIIDesensitizerIDCard</t>
+        </is>
+      </c>
+      <c r="C909" t="inlineStr">
+        <is>
+          <t>id_card_full_mask</t>
+        </is>
+      </c>
+      <c r="D909" t="inlineStr">
+        <is>
+          <t>身份证 full 遮蔽</t>
+        </is>
+      </c>
+    </row>
+    <row r="910">
+      <c r="A910" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B910" t="inlineStr">
+        <is>
+          <t>TestPIIDesensitizerEmail</t>
+        </is>
+      </c>
+      <c r="C910" t="inlineStr">
+        <is>
+          <t>email_partial_mask</t>
+        </is>
+      </c>
+      <c r="D910" t="inlineStr">
+        <is>
+          <t>邮箱 partial 遮蔽</t>
+        </is>
+      </c>
+    </row>
+    <row r="911">
+      <c r="A911" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B911" t="inlineStr">
+        <is>
+          <t>TestPIIDesensitizerEmail</t>
+        </is>
+      </c>
+      <c r="C911" t="inlineStr">
+        <is>
+          <t>email_short_prefix</t>
+        </is>
+      </c>
+      <c r="D911" t="inlineStr">
+        <is>
+          <t>短前缀邮箱遮蔽</t>
+        </is>
+      </c>
+    </row>
+    <row r="912">
+      <c r="A912" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B912" t="inlineStr">
+        <is>
+          <t>TestPIIDesensitizerEmail</t>
+        </is>
+      </c>
+      <c r="C912" t="inlineStr">
+        <is>
+          <t>email_full_mask</t>
+        </is>
+      </c>
+      <c r="D912" t="inlineStr">
+        <is>
+          <t>邮箱 full 遮蔽</t>
+        </is>
+      </c>
+    </row>
+    <row r="913">
+      <c r="A913" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B913" t="inlineStr">
+        <is>
+          <t>TestPIIDesensitizerAPIKey</t>
+        </is>
+      </c>
+      <c r="C913" t="inlineStr">
+        <is>
+          <t>openai_api_key_partial</t>
+        </is>
+      </c>
+      <c r="D913" t="inlineStr">
+        <is>
+          <t>OpenAI API Key partial 遮蔽</t>
+        </is>
+      </c>
+    </row>
+    <row r="914">
+      <c r="A914" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B914" t="inlineStr">
+        <is>
+          <t>TestPIIDesensitizerAPIKey</t>
+        </is>
+      </c>
+      <c r="C914" t="inlineStr">
+        <is>
+          <t>bearer_token</t>
+        </is>
+      </c>
+      <c r="D914" t="inlineStr">
+        <is>
+          <t>Bearer token 遮蔽</t>
+        </is>
+      </c>
+    </row>
+    <row r="915">
+      <c r="A915" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B915" t="inlineStr">
+        <is>
+          <t>TestPIIDesensitizerAPIKey</t>
+        </is>
+      </c>
+      <c r="C915" t="inlineStr">
+        <is>
+          <t>github_pat</t>
+        </is>
+      </c>
+      <c r="D915" t="inlineStr">
+        <is>
+          <t>GitHub PAT 遮蔽</t>
+        </is>
+      </c>
+    </row>
+    <row r="916">
+      <c r="A916" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B916" t="inlineStr">
+        <is>
+          <t>TestPIIDesensitizerAPIKey</t>
+        </is>
+      </c>
+      <c r="C916" t="inlineStr">
+        <is>
+          <t>aws_key</t>
+        </is>
+      </c>
+      <c r="D916" t="inlineStr">
+        <is>
+          <t>AWS Key 遮蔽</t>
+        </is>
+      </c>
+    </row>
+    <row r="917">
+      <c r="A917" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B917" t="inlineStr">
+        <is>
+          <t>TestPIIDesensitizerMixed</t>
+        </is>
+      </c>
+      <c r="C917" t="inlineStr">
+        <is>
+          <t>multiple_pii_types</t>
+        </is>
+      </c>
+      <c r="D917" t="inlineStr">
+        <is>
+          <t>多种 PII 同时遮蔽</t>
+        </is>
+      </c>
+    </row>
+    <row r="918">
+      <c r="A918" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B918" t="inlineStr">
+        <is>
+          <t>TestPIIDesensitizerMixed</t>
+        </is>
+      </c>
+      <c r="C918" t="inlineStr">
+        <is>
+          <t>selective_pii_types</t>
+        </is>
+      </c>
+      <c r="D918" t="inlineStr">
+        <is>
+          <t>选择性启用 PII 类型</t>
+        </is>
+      </c>
+    </row>
+    <row r="919">
+      <c r="A919" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B919" t="inlineStr">
+        <is>
+          <t>TestPIIDesensitizerMixed</t>
+        </is>
+      </c>
+      <c r="C919" t="inlineStr">
+        <is>
+          <t>no_pii_in_text</t>
+        </is>
+      </c>
+      <c r="D919" t="inlineStr">
+        <is>
+          <t>无 PII 时不遮蔽</t>
+        </is>
+      </c>
+    </row>
+    <row r="920">
+      <c r="A920" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B920" t="inlineStr">
+        <is>
+          <t>TestPIIDesensitizerMixed</t>
+        </is>
+      </c>
+      <c r="C920" t="inlineStr">
+        <is>
+          <t>custom_mask_char</t>
+        </is>
+      </c>
+      <c r="D920" t="inlineStr">
+        <is>
+          <t>自定义遮蔽字符</t>
+        </is>
+      </c>
+    </row>
+    <row r="921">
+      <c r="A921" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B921" t="inlineStr">
+        <is>
+          <t>TestPIIDesensitizerDisabled</t>
+        </is>
+      </c>
+      <c r="C921" t="inlineStr">
+        <is>
+          <t>pii_disabled_no_masking</t>
+        </is>
+      </c>
+      <c r="D921" t="inlineStr">
+        <is>
+          <t>PII 禁用时不遮蔽</t>
+        </is>
+      </c>
+    </row>
+    <row r="922">
+      <c r="A922" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B922" t="inlineStr">
+        <is>
+          <t>TestPIIConfig</t>
+        </is>
+      </c>
+      <c r="C922" t="inlineStr">
+        <is>
+          <t>default_pii_disabled</t>
+        </is>
+      </c>
+      <c r="D922" t="inlineStr">
+        <is>
+          <t>默认 PII 禁用</t>
+        </is>
+      </c>
+    </row>
+    <row r="923">
+      <c r="A923" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B923" t="inlineStr">
+        <is>
+          <t>TestPIIConfig</t>
+        </is>
+      </c>
+      <c r="C923" t="inlineStr">
+        <is>
+          <t>pii_config_fields</t>
+        </is>
+      </c>
+      <c r="D923" t="inlineStr">
+        <is>
+          <t>PII 配置字段正确</t>
+        </is>
+      </c>
+    </row>
+    <row r="924">
+      <c r="A924" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B924" t="inlineStr">
+        <is>
+          <t>TestPIIConfig</t>
+        </is>
+      </c>
+      <c r="C924" t="inlineStr">
+        <is>
+          <t>pii_types_default</t>
+        </is>
+      </c>
+      <c r="D924" t="inlineStr">
+        <is>
+          <t>PII 默认类型列表</t>
+        </is>
+      </c>
+    </row>
+    <row r="925">
+      <c r="A925" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B925" t="inlineStr">
+        <is>
+          <t>TestPIIConfig</t>
+        </is>
+      </c>
+      <c r="C925" t="inlineStr">
+        <is>
+          <t>pii_types_custom</t>
+        </is>
+      </c>
+      <c r="D925" t="inlineStr">
+        <is>
+          <t>自定义 PII 类型</t>
+        </is>
+      </c>
+    </row>
+    <row r="926">
+      <c r="A926" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B926" t="inlineStr">
+        <is>
+          <t>TestPIIConfig</t>
+        </is>
+      </c>
+      <c r="C926" t="inlineStr">
+        <is>
+          <t>config_from_dict_with_pii</t>
+        </is>
+      </c>
+      <c r="D926" t="inlineStr">
+        <is>
+          <t>_from_dict 反序列化 PII 配置</t>
+        </is>
+      </c>
+    </row>
+    <row r="927">
+      <c r="A927" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B927" t="inlineStr">
+        <is>
+          <t>TestPIISanitizerIntegration</t>
+        </is>
+      </c>
+      <c r="C927" t="inlineStr">
+        <is>
+          <t>pii_masked_before_injection_check</t>
+        </is>
+      </c>
+      <c r="D927" t="inlineStr">
+        <is>
+          <t>PII 在注入检查前遮蔽</t>
+        </is>
+      </c>
+    </row>
+    <row r="928">
+      <c r="A928" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B928" t="inlineStr">
+        <is>
+          <t>TestPIISanitizerIntegration</t>
+        </is>
+      </c>
+      <c r="C928" t="inlineStr">
+        <is>
+          <t>pii_actions_recorded</t>
+        </is>
+      </c>
+      <c r="D928" t="inlineStr">
+        <is>
+          <t>PII 遮蔽记录到 actions</t>
+        </is>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B929" t="inlineStr">
+        <is>
+          <t>TestPIISanitizerIntegration</t>
+        </is>
+      </c>
+      <c r="C929" t="inlineStr">
+        <is>
+          <t>pii_disabled_no_action</t>
+        </is>
+      </c>
+      <c r="D929" t="inlineStr">
+        <is>
+          <t>PII 禁用时无 action</t>
+        </is>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B930" t="inlineStr">
+        <is>
+          <t>TestPIISanitizerIntegration</t>
+        </is>
+      </c>
+      <c r="C930" t="inlineStr">
+        <is>
+          <t>pii_with_injection_both_detected</t>
+        </is>
+      </c>
+      <c r="D930" t="inlineStr">
+        <is>
+          <t>PII+注入同时存在时注入拒绝</t>
+        </is>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B931" t="inlineStr">
+        <is>
+          <t>TestPIISanitizerIntegration</t>
+        </is>
+      </c>
+      <c r="C931" t="inlineStr">
+        <is>
+          <t>pii_result_matches_populated</t>
+        </is>
+      </c>
+      <c r="D931" t="inlineStr">
+        <is>
+          <t>PII 结果填充 pii_matches</t>
+        </is>
+      </c>
+    </row>
+    <row r="932">
+      <c r="A932" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B932" t="inlineStr">
+        <is>
+          <t>TestPIISanitizerIntegration</t>
+        </is>
+      </c>
+      <c r="C932" t="inlineStr">
+        <is>
+          <t>rejected_result_has_empty_pii_matches</t>
+        </is>
+      </c>
+      <c r="D932" t="inlineStr">
+        <is>
+          <t>拒绝结果 pii_matches 为空</t>
+        </is>
+      </c>
+    </row>
+    <row r="933">
+      <c r="A933" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B933" t="inlineStr">
+        <is>
+          <t>TestPIIOrchestratorIntegration</t>
+        </is>
+      </c>
+      <c r="C933" t="inlineStr">
+        <is>
+          <t>orchestrator_masks_pii</t>
+        </is>
+      </c>
+      <c r="D933" t="inlineStr">
+        <is>
+          <t>orchestrator 遮蔽 PII</t>
+        </is>
+      </c>
+    </row>
+    <row r="934">
+      <c r="A934" t="inlineStr">
+        <is>
+          <t>sanitizer</t>
+        </is>
+      </c>
+      <c r="B934" t="inlineStr">
+        <is>
+          <t>TestPIIOrchestratorIntegration</t>
+        </is>
+      </c>
+      <c r="C934" t="inlineStr">
+        <is>
+          <t>orchestrator_pii_disabled</t>
+        </is>
+      </c>
+      <c r="D934" t="inlineStr">
+        <is>
+          <t>PII 禁用时 orchestrator 不遮蔽</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: v0.8.6 有害内容过滤 — 4 类检测 + block/warn/replace 动作 + 中间件
- 新增 HarmfulContentFilter: 输出侧有害内容过滤，与 OutputGuard 互补（防信息泄露 vs 防有害内容）
- 支持 violence/hate/dangerous/illegal 4 类检测，中英文正则模式
- 保守模式：仅匹配指令性短语（"如何制造"/"how to make"），避免误报
- 按 category 可配 block/warn/replace 动作，block 优先于 warn/replace
- 默认关闭（opt-in），有害内容定义因场景而异
- 新增 HarmfulContentMiddleware (priority=99) 扫描工具输出
- 新增 HarmfulContentFilterConfig 配置项 + CLI 集成
- 重构: 合并 _compiled_patterns/_custom_patterns 为单一 _patterns dict
- 清理: 移除 harmful_filter.py 中未使用的 TerminationReason 导入
- 文档: api.md/constraints.md/architecture.md/tutorial.md 补全 HarmfulContentFilter 说明
- 70 个测试用例，全量 1565 测试通过

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/test_cases.xlsx
+++ b/tests/test_cases.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1007"/>
+  <dimension ref="A1:E1077"/>
   <sheetFormatPr baseColWidth="15" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25197,6 +25197,1546 @@
         </is>
       </c>
     </row>
+    <row r="1008">
+      <c r="A1008" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1008" t="inlineStr">
+        <is>
+          <t>TestHarmfulContentFilterConfig:</t>
+        </is>
+      </c>
+      <c r="C1008" t="inlineStr">
+        <is>
+          <t>test_default_config_disabled</t>
+        </is>
+      </c>
+      <c r="D1008" t="inlineStr">
+        <is>
+          <t>test_default_config_disabled</t>
+        </is>
+      </c>
+    </row>
+    <row r="1009">
+      <c r="A1009" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1009" t="inlineStr">
+        <is>
+          <t>TestHarmfulContentFilterConfig:</t>
+        </is>
+      </c>
+      <c r="C1009" t="inlineStr">
+        <is>
+          <t>test_default_categories</t>
+        </is>
+      </c>
+      <c r="D1009" t="inlineStr">
+        <is>
+          <t>test_default_categories</t>
+        </is>
+      </c>
+    </row>
+    <row r="1010">
+      <c r="A1010" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1010" t="inlineStr">
+        <is>
+          <t>TestHarmfulContentFilterConfig:</t>
+        </is>
+      </c>
+      <c r="C1010" t="inlineStr">
+        <is>
+          <t>test_default_action_is_block</t>
+        </is>
+      </c>
+      <c r="D1010" t="inlineStr">
+        <is>
+          <t>test_default_action_is_block</t>
+        </is>
+      </c>
+    </row>
+    <row r="1011">
+      <c r="A1011" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1011" t="inlineStr">
+        <is>
+          <t>TestHarmfulContentFilterConfig:</t>
+        </is>
+      </c>
+      <c r="C1011" t="inlineStr">
+        <is>
+          <t>test_custom_config</t>
+        </is>
+      </c>
+      <c r="D1011" t="inlineStr">
+        <is>
+          <t>test_custom_config</t>
+        </is>
+      </c>
+    </row>
+    <row r="1012">
+      <c r="A1012" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1012" t="inlineStr">
+        <is>
+          <t>TestHarmfulContentFilterConfig:</t>
+        </is>
+      </c>
+      <c r="C1012" t="inlineStr">
+        <is>
+          <t>test_config_in_full_config</t>
+        </is>
+      </c>
+      <c r="D1012" t="inlineStr">
+        <is>
+          <t>test_config_in_full_config</t>
+        </is>
+      </c>
+    </row>
+    <row r="1013">
+      <c r="A1013" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1013" t="inlineStr">
+        <is>
+          <t>TestHarmfulContentFilterConfig:</t>
+        </is>
+      </c>
+      <c r="C1013" t="inlineStr">
+        <is>
+          <t>test_config_from_dict</t>
+        </is>
+      </c>
+      <c r="D1013" t="inlineStr">
+        <is>
+          <t>从字典创建配置</t>
+        </is>
+      </c>
+    </row>
+    <row r="1014">
+      <c r="A1014" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1014" t="inlineStr">
+        <is>
+          <t>TestHarmfulContentFilterConfig:</t>
+        </is>
+      </c>
+      <c r="C1014" t="inlineStr">
+        <is>
+          <t>test_custom_patterns</t>
+        </is>
+      </c>
+      <c r="D1014" t="inlineStr">
+        <is>
+          <t>test_custom_patterns</t>
+        </is>
+      </c>
+    </row>
+    <row r="1015">
+      <c r="A1015" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1015" t="inlineStr">
+        <is>
+          <t>TestHarmfulContentFilterConfig:</t>
+        </is>
+      </c>
+      <c r="C1015" t="inlineStr">
+        <is>
+          <t>test_category_actions</t>
+        </is>
+      </c>
+      <c r="D1015" t="inlineStr">
+        <is>
+          <t>test_category_actions</t>
+        </is>
+      </c>
+    </row>
+    <row r="1016">
+      <c r="A1016" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1016" t="inlineStr">
+        <is>
+          <t>TestHarmfulFilterResult:</t>
+        </is>
+      </c>
+      <c r="C1016" t="inlineStr">
+        <is>
+          <t>test_result_no_harmful</t>
+        </is>
+      </c>
+      <c r="D1016" t="inlineStr">
+        <is>
+          <t>test_result_no_harmful</t>
+        </is>
+      </c>
+    </row>
+    <row r="1017">
+      <c r="A1017" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1017" t="inlineStr">
+        <is>
+          <t>TestHarmfulFilterResult:</t>
+        </is>
+      </c>
+      <c r="C1017" t="inlineStr">
+        <is>
+          <t>test_result_blocked</t>
+        </is>
+      </c>
+      <c r="D1017" t="inlineStr">
+        <is>
+          <t>已拦截结果</t>
+        </is>
+      </c>
+    </row>
+    <row r="1018">
+      <c r="A1018" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1018" t="inlineStr">
+        <is>
+          <t>TestHarmfulFilterResult:</t>
+        </is>
+      </c>
+      <c r="C1018" t="inlineStr">
+        <is>
+          <t>test_result_warned</t>
+        </is>
+      </c>
+      <c r="D1018" t="inlineStr">
+        <is>
+          <t>已警告结果</t>
+        </is>
+      </c>
+    </row>
+    <row r="1019">
+      <c r="A1019" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1019" t="inlineStr">
+        <is>
+          <t>TestHarmfulFilterResult:</t>
+        </is>
+      </c>
+      <c r="C1019" t="inlineStr">
+        <is>
+          <t>test_result_replaced</t>
+        </is>
+      </c>
+      <c r="D1019" t="inlineStr">
+        <is>
+          <t>test_result_replaced</t>
+        </is>
+      </c>
+    </row>
+    <row r="1020">
+      <c r="A1020" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1020" t="inlineStr">
+        <is>
+          <t>TestViolenceDetection:</t>
+        </is>
+      </c>
+      <c r="C1020" t="inlineStr">
+        <is>
+          <t>test_bomb_making_english</t>
+        </is>
+      </c>
+      <c r="D1020" t="inlineStr">
+        <is>
+          <t>test_bomb_making_english</t>
+        </is>
+      </c>
+    </row>
+    <row r="1021">
+      <c r="A1021" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1021" t="inlineStr">
+        <is>
+          <t>TestViolenceDetection:</t>
+        </is>
+      </c>
+      <c r="C1021" t="inlineStr">
+        <is>
+          <t>test_weapon_making_english</t>
+        </is>
+      </c>
+      <c r="D1021" t="inlineStr">
+        <is>
+          <t>test_weapon_making_english</t>
+        </is>
+      </c>
+    </row>
+    <row r="1022">
+      <c r="A1022" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1022" t="inlineStr">
+        <is>
+          <t>TestViolenceDetection:</t>
+        </is>
+      </c>
+      <c r="C1022" t="inlineStr">
+        <is>
+          <t>test_bomb_making_chinese</t>
+        </is>
+      </c>
+      <c r="D1022" t="inlineStr">
+        <is>
+          <t>test_bomb_making_chinese</t>
+        </is>
+      </c>
+    </row>
+    <row r="1023">
+      <c r="A1023" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1023" t="inlineStr">
+        <is>
+          <t>TestViolenceDetection:</t>
+        </is>
+      </c>
+      <c r="C1023" t="inlineStr">
+        <is>
+          <t>test_weapon_chinese</t>
+        </is>
+      </c>
+      <c r="D1023" t="inlineStr">
+        <is>
+          <t>test_weapon_chinese</t>
+        </is>
+      </c>
+    </row>
+    <row r="1024">
+      <c r="A1024" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1024" t="inlineStr">
+        <is>
+          <t>TestViolenceDetection:</t>
+        </is>
+      </c>
+      <c r="C1024" t="inlineStr">
+        <is>
+          <t>test_no_violence_in_safe_text</t>
+        </is>
+      </c>
+      <c r="D1024" t="inlineStr">
+        <is>
+          <t>test_no_violence_in_safe_text</t>
+        </is>
+      </c>
+    </row>
+    <row r="1025">
+      <c r="A1025" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1025" t="inlineStr">
+        <is>
+          <t>TestHateDetection:</t>
+        </is>
+      </c>
+      <c r="C1025" t="inlineStr">
+        <is>
+          <t>test_hate_speech_english</t>
+        </is>
+      </c>
+      <c r="D1025" t="inlineStr">
+        <is>
+          <t>test_hate_speech_english</t>
+        </is>
+      </c>
+    </row>
+    <row r="1026">
+      <c r="A1026" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1026" t="inlineStr">
+        <is>
+          <t>TestHateDetection:</t>
+        </is>
+      </c>
+      <c r="C1026" t="inlineStr">
+        <is>
+          <t>test_hate_speech_chinese</t>
+        </is>
+      </c>
+      <c r="D1026" t="inlineStr">
+        <is>
+          <t>test_hate_speech_chinese</t>
+        </is>
+      </c>
+    </row>
+    <row r="1027">
+      <c r="A1027" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1027" t="inlineStr">
+        <is>
+          <t>TestHateDetection:</t>
+        </is>
+      </c>
+      <c r="C1027" t="inlineStr">
+        <is>
+          <t>test_no_hate_in_discussion</t>
+        </is>
+      </c>
+      <c r="D1027" t="inlineStr">
+        <is>
+          <t>test_no_hate_in_discussion</t>
+        </is>
+      </c>
+    </row>
+    <row r="1028">
+      <c r="A1028" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1028" t="inlineStr">
+        <is>
+          <t>TestDangerousDetection:</t>
+        </is>
+      </c>
+      <c r="C1028" t="inlineStr">
+        <is>
+          <t>test_suicide_methods_english</t>
+        </is>
+      </c>
+      <c r="D1028" t="inlineStr">
+        <is>
+          <t>test_suicide_methods_english</t>
+        </is>
+      </c>
+    </row>
+    <row r="1029">
+      <c r="A1029" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1029" t="inlineStr">
+        <is>
+          <t>TestDangerousDetection:</t>
+        </is>
+      </c>
+      <c r="C1029" t="inlineStr">
+        <is>
+          <t>test_suicide_methods_chinese</t>
+        </is>
+      </c>
+      <c r="D1029" t="inlineStr">
+        <is>
+          <t>test_suicide_methods_chinese</t>
+        </is>
+      </c>
+    </row>
+    <row r="1030">
+      <c r="A1030" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1030" t="inlineStr">
+        <is>
+          <t>TestDangerousDetection:</t>
+        </is>
+      </c>
+      <c r="C1030" t="inlineStr">
+        <is>
+          <t>test_drug_synthesis_english</t>
+        </is>
+      </c>
+      <c r="D1030" t="inlineStr">
+        <is>
+          <t>test_drug_synthesis_english</t>
+        </is>
+      </c>
+    </row>
+    <row r="1031">
+      <c r="A1031" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1031" t="inlineStr">
+        <is>
+          <t>TestDangerousDetection:</t>
+        </is>
+      </c>
+      <c r="C1031" t="inlineStr">
+        <is>
+          <t>test_hacking_instructions_english</t>
+        </is>
+      </c>
+      <c r="D1031" t="inlineStr">
+        <is>
+          <t>test_hacking_instructions_english</t>
+        </is>
+      </c>
+    </row>
+    <row r="1032">
+      <c r="A1032" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1032" t="inlineStr">
+        <is>
+          <t>TestDangerousDetection:</t>
+        </is>
+      </c>
+      <c r="C1032" t="inlineStr">
+        <is>
+          <t>test_no_dangerous_in_safe_text</t>
+        </is>
+      </c>
+      <c r="D1032" t="inlineStr">
+        <is>
+          <t>test_no_dangerous_in_safe_text</t>
+        </is>
+      </c>
+    </row>
+    <row r="1033">
+      <c r="A1033" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1033" t="inlineStr">
+        <is>
+          <t>TestIllegalDetection:</t>
+        </is>
+      </c>
+      <c r="C1033" t="inlineStr">
+        <is>
+          <t>test_money_laundering_english</t>
+        </is>
+      </c>
+      <c r="D1033" t="inlineStr">
+        <is>
+          <t>test_money_laundering_english</t>
+        </is>
+      </c>
+    </row>
+    <row r="1034">
+      <c r="A1034" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1034" t="inlineStr">
+        <is>
+          <t>TestIllegalDetection:</t>
+        </is>
+      </c>
+      <c r="C1034" t="inlineStr">
+        <is>
+          <t>test_forgery_instructions_english</t>
+        </is>
+      </c>
+      <c r="D1034" t="inlineStr">
+        <is>
+          <t>test_forgery_instructions_english</t>
+        </is>
+      </c>
+    </row>
+    <row r="1035">
+      <c r="A1035" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1035" t="inlineStr">
+        <is>
+          <t>TestIllegalDetection:</t>
+        </is>
+      </c>
+      <c r="C1035" t="inlineStr">
+        <is>
+          <t>test_money_laundering_chinese</t>
+        </is>
+      </c>
+      <c r="D1035" t="inlineStr">
+        <is>
+          <t>test_money_laundering_chinese</t>
+        </is>
+      </c>
+    </row>
+    <row r="1036">
+      <c r="A1036" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1036" t="inlineStr">
+        <is>
+          <t>TestIllegalDetection:</t>
+        </is>
+      </c>
+      <c r="C1036" t="inlineStr">
+        <is>
+          <t>test_no_illegal_in_safe_text</t>
+        </is>
+      </c>
+      <c r="D1036" t="inlineStr">
+        <is>
+          <t>test_no_illegal_in_safe_text</t>
+        </is>
+      </c>
+    </row>
+    <row r="1037">
+      <c r="A1037" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1037" t="inlineStr">
+        <is>
+          <t>TestBlocking:</t>
+        </is>
+      </c>
+      <c r="C1037" t="inlineStr">
+        <is>
+          <t>test_block_action_blocks_response</t>
+        </is>
+      </c>
+      <c r="D1037" t="inlineStr">
+        <is>
+          <t>test_block_action_blocks_response</t>
+        </is>
+      </c>
+    </row>
+    <row r="1038">
+      <c r="A1038" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1038" t="inlineStr">
+        <is>
+          <t>TestBlocking:</t>
+        </is>
+      </c>
+      <c r="C1038" t="inlineStr">
+        <is>
+          <t>test_block_emits_events</t>
+        </is>
+      </c>
+      <c r="D1038" t="inlineStr">
+        <is>
+          <t>test_block_emits_events</t>
+        </is>
+      </c>
+    </row>
+    <row r="1039">
+      <c r="A1039" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1039" t="inlineStr">
+        <is>
+          <t>TestBlocking:</t>
+        </is>
+      </c>
+      <c r="C1039" t="inlineStr">
+        <is>
+          <t>test_blocked_response_is_empty</t>
+        </is>
+      </c>
+      <c r="D1039" t="inlineStr">
+        <is>
+          <t>test_blocked_response_is_empty</t>
+        </is>
+      </c>
+    </row>
+    <row r="1040">
+      <c r="A1040" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1040" t="inlineStr">
+        <is>
+          <t>TestBlocking:</t>
+        </is>
+      </c>
+      <c r="C1040" t="inlineStr">
+        <is>
+          <t>test_block_reason_includes_categories</t>
+        </is>
+      </c>
+      <c r="D1040" t="inlineStr">
+        <is>
+          <t>test_block_reason_includes_categories</t>
+        </is>
+      </c>
+    </row>
+    <row r="1041">
+      <c r="A1041" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1041" t="inlineStr">
+        <is>
+          <t>TestWarning:</t>
+        </is>
+      </c>
+      <c r="C1041" t="inlineStr">
+        <is>
+          <t>test_warn_action_does_not_block</t>
+        </is>
+      </c>
+      <c r="D1041" t="inlineStr">
+        <is>
+          <t>test_warn_action_does_not_block</t>
+        </is>
+      </c>
+    </row>
+    <row r="1042">
+      <c r="A1042" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1042" t="inlineStr">
+        <is>
+          <t>TestWarning:</t>
+        </is>
+      </c>
+      <c r="C1042" t="inlineStr">
+        <is>
+          <t>test_warn_prepend_notice</t>
+        </is>
+      </c>
+      <c r="D1042" t="inlineStr">
+        <is>
+          <t>test_warn_prepend_notice</t>
+        </is>
+      </c>
+    </row>
+    <row r="1043">
+      <c r="A1043" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1043" t="inlineStr">
+        <is>
+          <t>TestWarning:</t>
+        </is>
+      </c>
+      <c r="C1043" t="inlineStr">
+        <is>
+          <t>test_warn_does_not_remove_text</t>
+        </is>
+      </c>
+      <c r="D1043" t="inlineStr">
+        <is>
+          <t>test_warn_does_not_remove_text</t>
+        </is>
+      </c>
+    </row>
+    <row r="1044">
+      <c r="A1044" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1044" t="inlineStr">
+        <is>
+          <t>TestReplacement:</t>
+        </is>
+      </c>
+      <c r="C1044" t="inlineStr">
+        <is>
+          <t>test_replace_action_substitutes_text</t>
+        </is>
+      </c>
+      <c r="D1044" t="inlineStr">
+        <is>
+          <t>test_replace_action_substitutes_text</t>
+        </is>
+      </c>
+    </row>
+    <row r="1045">
+      <c r="A1045" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1045" t="inlineStr">
+        <is>
+          <t>TestReplacement:</t>
+        </is>
+      </c>
+      <c r="C1045" t="inlineStr">
+        <is>
+          <t>test_custom_replacement_text</t>
+        </is>
+      </c>
+      <c r="D1045" t="inlineStr">
+        <is>
+          <t>test_custom_replacement_text</t>
+        </is>
+      </c>
+    </row>
+    <row r="1046">
+      <c r="A1046" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1046" t="inlineStr">
+        <is>
+          <t>TestReplacement:</t>
+        </is>
+      </c>
+      <c r="C1046" t="inlineStr">
+        <is>
+          <t>test_multiple_replacements</t>
+        </is>
+      </c>
+      <c r="D1046" t="inlineStr">
+        <is>
+          <t>test_multiple_replacements</t>
+        </is>
+      </c>
+    </row>
+    <row r="1047">
+      <c r="A1047" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1047" t="inlineStr">
+        <is>
+          <t>TestCategoryActions:</t>
+        </is>
+      </c>
+      <c r="C1047" t="inlineStr">
+        <is>
+          <t>test_different_actions_per_category</t>
+        </is>
+      </c>
+      <c r="D1047" t="inlineStr">
+        <is>
+          <t>test_different_actions_per_category</t>
+        </is>
+      </c>
+    </row>
+    <row r="1048">
+      <c r="A1048" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1048" t="inlineStr">
+        <is>
+          <t>TestCategoryActions:</t>
+        </is>
+      </c>
+      <c r="C1048" t="inlineStr">
+        <is>
+          <t>test_category_action_overrides_default</t>
+        </is>
+      </c>
+      <c r="D1048" t="inlineStr">
+        <is>
+          <t>test_category_action_overrides_default</t>
+        </is>
+      </c>
+    </row>
+    <row r="1049">
+      <c r="A1049" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1049" t="inlineStr">
+        <is>
+          <t>TestCategoryActions:</t>
+        </is>
+      </c>
+      <c r="C1049" t="inlineStr">
+        <is>
+          <t>test_mixed_actions_block_takes_precedence</t>
+        </is>
+      </c>
+      <c r="D1049" t="inlineStr">
+        <is>
+          <t>test_mixed_actions_block_takes_precedence</t>
+        </is>
+      </c>
+    </row>
+    <row r="1050">
+      <c r="A1050" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1050" t="inlineStr">
+        <is>
+          <t>TestOrchestratorIntegration:</t>
+        </is>
+      </c>
+      <c r="C1050" t="inlineStr">
+        <is>
+          <t>test_orchestrator_blocks_harmful_output</t>
+        </is>
+      </c>
+      <c r="D1050" t="inlineStr">
+        <is>
+          <t>test_orchestrator_blocks_harmful_output</t>
+        </is>
+      </c>
+    </row>
+    <row r="1051">
+      <c r="A1051" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1051" t="inlineStr">
+        <is>
+          <t>TestOrchestratorIntegration:</t>
+        </is>
+      </c>
+      <c r="C1051" t="inlineStr">
+        <is>
+          <t>test_orchestrator_warns_harmful_output</t>
+        </is>
+      </c>
+      <c r="D1051" t="inlineStr">
+        <is>
+          <t>test_orchestrator_warns_harmful_output</t>
+        </is>
+      </c>
+    </row>
+    <row r="1052">
+      <c r="A1052" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1052" t="inlineStr">
+        <is>
+          <t>TestOrchestratorIntegration:</t>
+        </is>
+      </c>
+      <c r="C1052" t="inlineStr">
+        <is>
+          <t>test_orchestrator_replaces_harmful_output</t>
+        </is>
+      </c>
+      <c r="D1052" t="inlineStr">
+        <is>
+          <t>test_orchestrator_replaces_harmful_output</t>
+        </is>
+      </c>
+    </row>
+    <row r="1053">
+      <c r="A1053" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1053" t="inlineStr">
+        <is>
+          <t>TestOrchestratorIntegration:</t>
+        </is>
+      </c>
+      <c r="C1053" t="inlineStr">
+        <is>
+          <t>test_orchestrator_no_filter</t>
+        </is>
+      </c>
+      <c r="D1053" t="inlineStr">
+        <is>
+          <t>无过滤器</t>
+        </is>
+      </c>
+    </row>
+    <row r="1054">
+      <c r="A1054" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1054" t="inlineStr">
+        <is>
+          <t>TestOrchestratorIntegration:</t>
+        </is>
+      </c>
+      <c r="C1054" t="inlineStr">
+        <is>
+          <t>test_orchestrator_filter_disabled</t>
+        </is>
+      </c>
+      <c r="D1054" t="inlineStr">
+        <is>
+          <t>过滤器禁用</t>
+        </is>
+      </c>
+    </row>
+    <row r="1055">
+      <c r="A1055" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1055" t="inlineStr">
+        <is>
+          <t>TestOrchestratorIntegration:</t>
+        </is>
+      </c>
+      <c r="C1055" t="inlineStr">
+        <is>
+          <t>test_orchestrator_clean_output</t>
+        </is>
+      </c>
+      <c r="D1055" t="inlineStr">
+        <is>
+          <t>test_orchestrator_clean_output</t>
+        </is>
+      </c>
+    </row>
+    <row r="1056">
+      <c r="A1056" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1056" t="inlineStr">
+        <is>
+          <t>TestOrchestratorIntegration:</t>
+        </is>
+      </c>
+      <c r="C1056" t="inlineStr">
+        <is>
+          <t>test_orchestrator_filter_after_output_guard</t>
+        </is>
+      </c>
+      <c r="D1056" t="inlineStr">
+        <is>
+          <t>test_orchestrator_filter_after_output_guard</t>
+        </is>
+      </c>
+    </row>
+    <row r="1057">
+      <c r="A1057" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1057" t="inlineStr">
+        <is>
+          <t>TestHarmfulContentMiddleware:</t>
+        </is>
+      </c>
+      <c r="C1057" t="inlineStr">
+        <is>
+          <t>test_middleware_replaces_output</t>
+        </is>
+      </c>
+      <c r="D1057" t="inlineStr">
+        <is>
+          <t>test_middleware_replaces_output</t>
+        </is>
+      </c>
+    </row>
+    <row r="1058">
+      <c r="A1058" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1058" t="inlineStr">
+        <is>
+          <t>TestHarmfulContentMiddleware:</t>
+        </is>
+      </c>
+      <c r="C1058" t="inlineStr">
+        <is>
+          <t>test_middleware_no_filter</t>
+        </is>
+      </c>
+      <c r="D1058" t="inlineStr">
+        <is>
+          <t>中间件无过滤器</t>
+        </is>
+      </c>
+    </row>
+    <row r="1059">
+      <c r="A1059" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1059" t="inlineStr">
+        <is>
+          <t>TestHarmfulContentMiddleware:</t>
+        </is>
+      </c>
+      <c r="C1059" t="inlineStr">
+        <is>
+          <t>test_middleware_filter_disabled</t>
+        </is>
+      </c>
+      <c r="D1059" t="inlineStr">
+        <is>
+          <t>test_middleware_filter_disabled</t>
+        </is>
+      </c>
+    </row>
+    <row r="1060">
+      <c r="A1060" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1060" t="inlineStr">
+        <is>
+          <t>TestHarmfulContentMiddleware:</t>
+        </is>
+      </c>
+      <c r="C1060" t="inlineStr">
+        <is>
+          <t>test_middleware_no_harmful_data</t>
+        </is>
+      </c>
+      <c r="D1060" t="inlineStr">
+        <is>
+          <t>test_middleware_no_harmful_data</t>
+        </is>
+      </c>
+    </row>
+    <row r="1061">
+      <c r="A1061" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1061" t="inlineStr">
+        <is>
+          <t>TestHarmfulContentMiddleware:</t>
+        </is>
+      </c>
+      <c r="C1061" t="inlineStr">
+        <is>
+          <t>test_middleware_failed_result_skipped</t>
+        </is>
+      </c>
+      <c r="D1061" t="inlineStr">
+        <is>
+          <t>test_middleware_failed_result_skipped</t>
+        </is>
+      </c>
+    </row>
+    <row r="1062">
+      <c r="A1062" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1062" t="inlineStr">
+        <is>
+          <t>TestHarmfulContentMiddleware:</t>
+        </is>
+      </c>
+      <c r="C1062" t="inlineStr">
+        <is>
+          <t>test_middleware_priority</t>
+        </is>
+      </c>
+      <c r="D1062" t="inlineStr">
+        <is>
+          <t>test_middleware_priority</t>
+        </is>
+      </c>
+    </row>
+    <row r="1063">
+      <c r="A1063" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1063" t="inlineStr">
+        <is>
+          <t>TestCustomPatterns:</t>
+        </is>
+      </c>
+      <c r="C1063" t="inlineStr">
+        <is>
+          <t>test_custom_pattern_matches</t>
+        </is>
+      </c>
+      <c r="D1063" t="inlineStr">
+        <is>
+          <t>test_custom_pattern_matches</t>
+        </is>
+      </c>
+    </row>
+    <row r="1064">
+      <c r="A1064" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1064" t="inlineStr">
+        <is>
+          <t>TestCustomPatterns:</t>
+        </is>
+      </c>
+      <c r="C1064" t="inlineStr">
+        <is>
+          <t>test_custom_pattern_blocked</t>
+        </is>
+      </c>
+      <c r="D1064" t="inlineStr">
+        <is>
+          <t>test_custom_pattern_blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="1065">
+      <c r="A1065" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1065" t="inlineStr">
+        <is>
+          <t>TestCustomPatterns:</t>
+        </is>
+      </c>
+      <c r="C1065" t="inlineStr">
+        <is>
+          <t>test_invalid_custom_pattern_ignored</t>
+        </is>
+      </c>
+      <c r="D1065" t="inlineStr">
+        <is>
+          <t>test_invalid_custom_pattern_ignored</t>
+        </is>
+      </c>
+    </row>
+    <row r="1066">
+      <c r="A1066" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1066" t="inlineStr">
+        <is>
+          <t>TestCustomPatterns:</t>
+        </is>
+      </c>
+      <c r="C1066" t="inlineStr">
+        <is>
+          <t>test_custom_pattern_category_action</t>
+        </is>
+      </c>
+      <c r="D1066" t="inlineStr">
+        <is>
+          <t>test_custom_pattern_category_action</t>
+        </is>
+      </c>
+    </row>
+    <row r="1067">
+      <c r="A1067" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1067" t="inlineStr">
+        <is>
+          <t>TestEdgeCases:</t>
+        </is>
+      </c>
+      <c r="C1067" t="inlineStr">
+        <is>
+          <t>test_empty_input</t>
+        </is>
+      </c>
+      <c r="D1067" t="inlineStr">
+        <is>
+          <t>空输入</t>
+        </is>
+      </c>
+    </row>
+    <row r="1068">
+      <c r="A1068" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1068" t="inlineStr">
+        <is>
+          <t>TestEdgeCases:</t>
+        </is>
+      </c>
+      <c r="C1068" t="inlineStr">
+        <is>
+          <t>test_no_harmful_data</t>
+        </is>
+      </c>
+      <c r="D1068" t="inlineStr">
+        <is>
+          <t>test_no_harmful_data</t>
+        </is>
+      </c>
+    </row>
+    <row r="1069">
+      <c r="A1069" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1069" t="inlineStr">
+        <is>
+          <t>TestEdgeCases:</t>
+        </is>
+      </c>
+      <c r="C1069" t="inlineStr">
+        <is>
+          <t>test_multiple_categories_in_same_output</t>
+        </is>
+      </c>
+      <c r="D1069" t="inlineStr">
+        <is>
+          <t>test_multiple_categories_in_same_output</t>
+        </is>
+      </c>
+    </row>
+    <row r="1070">
+      <c r="A1070" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1070" t="inlineStr">
+        <is>
+          <t>TestEdgeCases:</t>
+        </is>
+      </c>
+      <c r="C1070" t="inlineStr">
+        <is>
+          <t>test_filter_disabled</t>
+        </is>
+      </c>
+      <c r="D1070" t="inlineStr">
+        <is>
+          <t>test_filter_disabled</t>
+        </is>
+      </c>
+    </row>
+    <row r="1071">
+      <c r="A1071" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1071" t="inlineStr">
+        <is>
+          <t>TestEdgeCases:</t>
+        </is>
+      </c>
+      <c r="C1071" t="inlineStr">
+        <is>
+          <t>test_scan_tool_output</t>
+        </is>
+      </c>
+      <c r="D1071" t="inlineStr">
+        <is>
+          <t>test_scan_tool_output</t>
+        </is>
+      </c>
+    </row>
+    <row r="1072">
+      <c r="A1072" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1072" t="inlineStr">
+        <is>
+          <t>TestEdgeCases:</t>
+        </is>
+      </c>
+      <c r="C1072" t="inlineStr">
+        <is>
+          <t>test_scan_tool_output_no_harmful</t>
+        </is>
+      </c>
+      <c r="D1072" t="inlineStr">
+        <is>
+          <t>test_scan_tool_output_no_harmful</t>
+        </is>
+      </c>
+    </row>
+    <row r="1073">
+      <c r="A1073" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1073" t="inlineStr">
+        <is>
+          <t>TestEdgeCases:</t>
+        </is>
+      </c>
+      <c r="C1073" t="inlineStr">
+        <is>
+          <t>test_unicode_output</t>
+        </is>
+      </c>
+      <c r="D1073" t="inlineStr">
+        <is>
+          <t>test_unicode_output</t>
+        </is>
+      </c>
+    </row>
+    <row r="1074">
+      <c r="A1074" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1074" t="inlineStr">
+        <is>
+          <t>TestEdgeCases:</t>
+        </is>
+      </c>
+      <c r="C1074" t="inlineStr">
+        <is>
+          <t>test_very_long_output</t>
+        </is>
+      </c>
+      <c r="D1074" t="inlineStr">
+        <is>
+          <t>超长输出</t>
+        </is>
+      </c>
+    </row>
+    <row r="1075">
+      <c r="A1075" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1075" t="inlineStr">
+        <is>
+          <t>TestSummarizeHarmfulMatches:</t>
+        </is>
+      </c>
+      <c r="C1075" t="inlineStr">
+        <is>
+          <t>test_empty_matches</t>
+        </is>
+      </c>
+      <c r="D1075" t="inlineStr">
+        <is>
+          <t>test_empty_matches</t>
+        </is>
+      </c>
+    </row>
+    <row r="1076">
+      <c r="A1076" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1076" t="inlineStr">
+        <is>
+          <t>TestSummarizeHarmfulMatches:</t>
+        </is>
+      </c>
+      <c r="C1076" t="inlineStr">
+        <is>
+          <t>test_single_category</t>
+        </is>
+      </c>
+      <c r="D1076" t="inlineStr">
+        <is>
+          <t>test_single_category</t>
+        </is>
+      </c>
+    </row>
+    <row r="1077">
+      <c r="A1077" t="inlineStr">
+        <is>
+          <t>harmful_filter</t>
+        </is>
+      </c>
+      <c r="B1077" t="inlineStr">
+        <is>
+          <t>TestSummarizeHarmfulMatches:</t>
+        </is>
+      </c>
+      <c r="C1077" t="inlineStr">
+        <is>
+          <t>test_multiple_categories</t>
+        </is>
+      </c>
+      <c r="D1077" t="inlineStr">
+        <is>
+          <t>多类别匹配</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: v0.8.7 结果正确性验证 — file_exists/code_syntax/command_success + block/warn/annotate
- 新增 ResultValidator: 输出侧结果正确性验证，在 OutputGuard 和 HarmfulContentFilter 之后执行
- 支持 file_exists/code_syntax/command_success 3 类验证检查，中英文正则模式
- file_exists: 验证声称创建的文件路径是否存在 (high severity)
- code_syntax: 验证声称正确的 Python/JSON/YAML 代码是否可编译/解析 (medium severity)
- command_success: 检查声称成功的命令输出中是否有矛盾的非零退出码 (high/low severity)
- 按 on_fail 配置 block/warn/annotate 动作，block 仅拦截 high-severity 失败
- 默认关闭（opt-in），验证仅标记明确可验证的声明，避免误报
- 新增 ResultValidatorConfig 配置项 + CLI 集成（拦截提示、结果通知、配置显示）
- 新增 TerminationReason.VALIDATION_FAILED + AgentEvent.VALIDATION_FAILED
- Orchestrator 管线新增 validator 步骤 + Builder 创建/传递 validator
- 文档: api.md/constraints.md/architecture.md/tutorial.md 补全 ResultValidator 说明
- 57 个测试用例，全量 1622 测试通过

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/test_cases.xlsx
+++ b/tests/test_cases.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1077"/>
+  <dimension ref="A1:E1134"/>
   <sheetFormatPr baseColWidth="15" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26737,6 +26737,1260 @@
         </is>
       </c>
     </row>
+    <row r="1078">
+      <c r="A1078" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1078" t="inlineStr">
+        <is>
+          <t>TestValidationCheck:</t>
+        </is>
+      </c>
+      <c r="C1078" t="inlineStr">
+        <is>
+          <t>test_creation</t>
+        </is>
+      </c>
+      <c r="D1078" t="inlineStr">
+        <is>
+          <t>ValidationCheck 创建与默认 severity</t>
+        </is>
+      </c>
+    </row>
+    <row r="1079">
+      <c r="A1079" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1079" t="inlineStr">
+        <is>
+          <t>TestValidationCheck:</t>
+        </is>
+      </c>
+      <c r="C1079" t="inlineStr">
+        <is>
+          <t>test_severity_override</t>
+        </is>
+      </c>
+      <c r="D1079" t="inlineStr">
+        <is>
+          <t>ValidationCheck severity 覆盖默认值</t>
+        </is>
+      </c>
+    </row>
+    <row r="1080">
+      <c r="A1080" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1080" t="inlineStr">
+        <is>
+          <t>TestValidationResult:</t>
+        </is>
+      </c>
+      <c r="C1080" t="inlineStr">
+        <is>
+          <t>test_no_checks</t>
+        </is>
+      </c>
+      <c r="D1080" t="inlineStr">
+        <is>
+          <t>ValidationResult 无检查项时不阻塞</t>
+        </is>
+      </c>
+    </row>
+    <row r="1081">
+      <c r="A1081" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1081" t="inlineStr">
+        <is>
+          <t>TestValidationResult:</t>
+        </is>
+      </c>
+      <c r="C1081" t="inlineStr">
+        <is>
+          <t>test_with_failed_checks</t>
+        </is>
+      </c>
+      <c r="D1081" t="inlineStr">
+        <is>
+          <t>ValidationResult 含失败检查项</t>
+        </is>
+      </c>
+    </row>
+    <row r="1082">
+      <c r="A1082" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1082" t="inlineStr">
+        <is>
+          <t>TestSummarizeValidationChecks:</t>
+        </is>
+      </c>
+      <c r="C1082" t="inlineStr">
+        <is>
+          <t>test_empty</t>
+        </is>
+      </c>
+      <c r="D1082" t="inlineStr">
+        <is>
+          <t>空检查列表摘要为空字符串</t>
+        </is>
+      </c>
+    </row>
+    <row r="1083">
+      <c r="A1083" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1083" t="inlineStr">
+        <is>
+          <t>TestSummarizeValidationChecks:</t>
+        </is>
+      </c>
+      <c r="C1083" t="inlineStr">
+        <is>
+          <t>test_single_type</t>
+        </is>
+      </c>
+      <c r="D1083" t="inlineStr">
+        <is>
+          <t>单类型检查摘要格式</t>
+        </is>
+      </c>
+    </row>
+    <row r="1084">
+      <c r="A1084" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1084" t="inlineStr">
+        <is>
+          <t>TestSummarizeValidationChecks:</t>
+        </is>
+      </c>
+      <c r="C1084" t="inlineStr">
+        <is>
+          <t>test_multiple_types</t>
+        </is>
+      </c>
+      <c r="D1084" t="inlineStr">
+        <is>
+          <t>多类型检查摘要格式含计数</t>
+        </is>
+      </c>
+    </row>
+    <row r="1085">
+      <c r="A1085" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1085" t="inlineStr">
+        <is>
+          <t>TestResultValidatorBasics:</t>
+        </is>
+      </c>
+      <c r="C1085" t="inlineStr">
+        <is>
+          <t>test_disabled_by_default</t>
+        </is>
+      </c>
+      <c r="D1085" t="inlineStr">
+        <is>
+          <t>ResultValidatorConfig 默认禁用</t>
+        </is>
+      </c>
+    </row>
+    <row r="1086">
+      <c r="A1086" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1086" t="inlineStr">
+        <is>
+          <t>TestResultValidatorBasics:</t>
+        </is>
+      </c>
+      <c r="C1086" t="inlineStr">
+        <is>
+          <t>test_enabled_property</t>
+        </is>
+      </c>
+      <c r="D1086" t="inlineStr">
+        <is>
+          <t>启用后 enabled 属性为 True</t>
+        </is>
+      </c>
+    </row>
+    <row r="1087">
+      <c r="A1087" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1087" t="inlineStr">
+        <is>
+          <t>TestResultValidatorBasics:</t>
+        </is>
+      </c>
+      <c r="C1087" t="inlineStr">
+        <is>
+          <t>test_disabled_validator_returns_unchanged</t>
+        </is>
+      </c>
+      <c r="D1087" t="inlineStr">
+        <is>
+          <t>禁用状态下验证器不修改输出</t>
+        </is>
+      </c>
+    </row>
+    <row r="1088">
+      <c r="A1088" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1088" t="inlineStr">
+        <is>
+          <t>TestResultValidatorBasics:</t>
+        </is>
+      </c>
+      <c r="C1088" t="inlineStr">
+        <is>
+          <t>test_scan_tool_output_returns_unchanged</t>
+        </is>
+      </c>
+      <c r="D1088" t="inlineStr">
+        <is>
+          <t>scan_tool_output 原样返回工具输出</t>
+        </is>
+      </c>
+    </row>
+    <row r="1089">
+      <c r="A1089" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1089" t="inlineStr">
+        <is>
+          <t>TestFileExistsCheck:</t>
+        </is>
+      </c>
+      <c r="C1089" t="inlineStr">
+        <is>
+          <t>test_file_exists_pass</t>
+        </is>
+      </c>
+      <c r="D1089" t="inlineStr">
+        <is>
+          <t>文件存在时检查通过</t>
+        </is>
+      </c>
+    </row>
+    <row r="1090">
+      <c r="A1090" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1090" t="inlineStr">
+        <is>
+          <t>TestFileExistsCheck:</t>
+        </is>
+      </c>
+      <c r="C1090" t="inlineStr">
+        <is>
+          <t>test_file_not_exists_fail</t>
+        </is>
+      </c>
+      <c r="D1090" t="inlineStr">
+        <is>
+          <t>文件不存在时检查失败</t>
+        </is>
+      </c>
+    </row>
+    <row r="1091">
+      <c r="A1091" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1091" t="inlineStr">
+        <is>
+          <t>TestFileExistsCheck:</t>
+        </is>
+      </c>
+      <c r="C1091" t="inlineStr">
+        <is>
+          <t>test_no_file_claims_no_checks</t>
+        </is>
+      </c>
+      <c r="D1091" t="inlineStr">
+        <is>
+          <t>无文件声明时不生成文件检查</t>
+        </is>
+      </c>
+    </row>
+    <row r="1092">
+      <c r="A1092" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1092" t="inlineStr">
+        <is>
+          <t>TestFileExistsCheck:</t>
+        </is>
+      </c>
+      <c r="C1092" t="inlineStr">
+        <is>
+          <t>test_url_paths_ignored</t>
+        </is>
+      </c>
+      <c r="D1092" t="inlineStr">
+        <is>
+          <t>URL 路径不被当作文件路径检查</t>
+        </is>
+      </c>
+    </row>
+    <row r="1093">
+      <c r="A1093" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1093" t="inlineStr">
+        <is>
+          <t>TestFileExistsCheck:</t>
+        </is>
+      </c>
+      <c r="C1093" t="inlineStr">
+        <is>
+          <t>test_file_claim_pattern_wrote</t>
+        </is>
+      </c>
+      <c r="D1093" t="inlineStr">
+        <is>
+          <t>wrote file 模式被检测</t>
+        </is>
+      </c>
+    </row>
+    <row r="1094">
+      <c r="A1094" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1094" t="inlineStr">
+        <is>
+          <t>TestFileExistsCheck:</t>
+        </is>
+      </c>
+      <c r="C1094" t="inlineStr">
+        <is>
+          <t>test_file_claim_pattern_saved_to</t>
+        </is>
+      </c>
+      <c r="D1094" t="inlineStr">
+        <is>
+          <t>saved to 模式被检测</t>
+        </is>
+      </c>
+    </row>
+    <row r="1095">
+      <c r="A1095" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1095" t="inlineStr">
+        <is>
+          <t>TestFileExistsCheck:</t>
+        </is>
+      </c>
+      <c r="C1095" t="inlineStr">
+        <is>
+          <t>test_file_claim_pattern_written_to</t>
+        </is>
+      </c>
+      <c r="D1095" t="inlineStr">
+        <is>
+          <t>written to 模式被检测</t>
+        </is>
+      </c>
+    </row>
+    <row r="1096">
+      <c r="A1096" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1096" t="inlineStr">
+        <is>
+          <t>TestFileExistsCheck:</t>
+        </is>
+      </c>
+      <c r="C1096" t="inlineStr">
+        <is>
+          <t>test_duplicate_paths_deduplicated</t>
+        </is>
+      </c>
+      <c r="D1096" t="inlineStr">
+        <is>
+          <t>重复路径只生成一次检查</t>
+        </is>
+      </c>
+    </row>
+    <row r="1097">
+      <c r="A1097" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1097" t="inlineStr">
+        <is>
+          <t>TestFileExistsCheck:</t>
+        </is>
+      </c>
+      <c r="C1097" t="inlineStr">
+        <is>
+          <t>test_file_exists_check_disabled</t>
+        </is>
+      </c>
+      <c r="D1097" t="inlineStr">
+        <is>
+          <t>file_exists 检查禁用时不生成文件检查</t>
+        </is>
+      </c>
+    </row>
+    <row r="1098">
+      <c r="A1098" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1098" t="inlineStr">
+        <is>
+          <t>TestCodeSyntaxCheck:</t>
+        </is>
+      </c>
+      <c r="C1098" t="inlineStr">
+        <is>
+          <t>test_valid_python_code_passes</t>
+        </is>
+      </c>
+      <c r="D1098" t="inlineStr">
+        <is>
+          <t>有效 Python 代码检查通过</t>
+        </is>
+      </c>
+    </row>
+    <row r="1099">
+      <c r="A1099" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1099" t="inlineStr">
+        <is>
+          <t>TestCodeSyntaxCheck:</t>
+        </is>
+      </c>
+      <c r="C1099" t="inlineStr">
+        <is>
+          <t>test_invalid_python_code_fails</t>
+        </is>
+      </c>
+      <c r="D1099" t="inlineStr">
+        <is>
+          <t>无效 Python 代码检查失败</t>
+        </is>
+      </c>
+    </row>
+    <row r="1100">
+      <c r="A1100" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1100" t="inlineStr">
+        <is>
+          <t>TestCodeSyntaxCheck:</t>
+        </is>
+      </c>
+      <c r="C1100" t="inlineStr">
+        <is>
+          <t>test_no_correctness_claim_no_check</t>
+        </is>
+      </c>
+      <c r="D1100" t="inlineStr">
+        <is>
+          <t>无正确性声明时不检查代码语法</t>
+        </is>
+      </c>
+    </row>
+    <row r="1101">
+      <c r="A1101" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1101" t="inlineStr">
+        <is>
+          <t>TestCodeSyntaxCheck:</t>
+        </is>
+      </c>
+      <c r="C1101" t="inlineStr">
+        <is>
+          <t>test_valid_json_passes</t>
+        </is>
+      </c>
+      <c r="D1101" t="inlineStr">
+        <is>
+          <t>有效 JSON 检查通过</t>
+        </is>
+      </c>
+    </row>
+    <row r="1102">
+      <c r="A1102" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1102" t="inlineStr">
+        <is>
+          <t>TestCodeSyntaxCheck:</t>
+        </is>
+      </c>
+      <c r="C1102" t="inlineStr">
+        <is>
+          <t>test_invalid_json_fails</t>
+        </is>
+      </c>
+      <c r="D1102" t="inlineStr">
+        <is>
+          <t>无效 JSON 检查失败</t>
+        </is>
+      </c>
+    </row>
+    <row r="1103">
+      <c r="A1103" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1103" t="inlineStr">
+        <is>
+          <t>TestCodeSyntaxCheck:</t>
+        </is>
+      </c>
+      <c r="C1103" t="inlineStr">
+        <is>
+          <t>test_code_syntax_check_disabled</t>
+        </is>
+      </c>
+      <c r="D1103" t="inlineStr">
+        <is>
+          <t>code_syntax 检查禁用时不生成代码检查</t>
+        </is>
+      </c>
+    </row>
+    <row r="1104">
+      <c r="A1104" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1104" t="inlineStr">
+        <is>
+          <t>TestCodeSyntaxCheck:</t>
+        </is>
+      </c>
+      <c r="C1104" t="inlineStr">
+        <is>
+          <t>test_syntax_error_detail_contains_line</t>
+        </is>
+      </c>
+      <c r="D1104" t="inlineStr">
+        <is>
+          <t>语法错误详情包含行号信息</t>
+        </is>
+      </c>
+    </row>
+    <row r="1105">
+      <c r="A1105" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1105" t="inlineStr">
+        <is>
+          <t>TestCodeSyntaxCheck:</t>
+        </is>
+      </c>
+      <c r="C1105" t="inlineStr">
+        <is>
+          <t>test_empty_code_block_ignored</t>
+        </is>
+      </c>
+      <c r="D1105" t="inlineStr">
+        <is>
+          <t>空代码块不生成检查</t>
+        </is>
+      </c>
+    </row>
+    <row r="1106">
+      <c r="A1106" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1106" t="inlineStr">
+        <is>
+          <t>TestCommandSuccessCheck:</t>
+        </is>
+      </c>
+      <c r="C1106" t="inlineStr">
+        <is>
+          <t>test_claim_with_zero_exit_code_passes</t>
+        </is>
+      </c>
+      <c r="D1106" t="inlineStr">
+        <is>
+          <t>退出码为 0 时命令成功检查通过</t>
+        </is>
+      </c>
+    </row>
+    <row r="1107">
+      <c r="A1107" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1107" t="inlineStr">
+        <is>
+          <t>TestCommandSuccessCheck:</t>
+        </is>
+      </c>
+      <c r="C1107" t="inlineStr">
+        <is>
+          <t>test_claim_with_nonzero_exit_code_fails</t>
+        </is>
+      </c>
+      <c r="D1107" t="inlineStr">
+        <is>
+          <t>退出码非 0 时命令成功检查失败</t>
+        </is>
+      </c>
+    </row>
+    <row r="1108">
+      <c r="A1108" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1108" t="inlineStr">
+        <is>
+          <t>TestCommandSuccessCheck:</t>
+        </is>
+      </c>
+      <c r="C1108" t="inlineStr">
+        <is>
+          <t>test_no_command_claim_no_check</t>
+        </is>
+      </c>
+      <c r="D1108" t="inlineStr">
+        <is>
+          <t>无命令成功声明时不检查</t>
+        </is>
+      </c>
+    </row>
+    <row r="1109">
+      <c r="A1109" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1109" t="inlineStr">
+        <is>
+          <t>TestCommandSuccessCheck:</t>
+        </is>
+      </c>
+      <c r="C1109" t="inlineStr">
+        <is>
+          <t>test_command_success_check_disabled</t>
+        </is>
+      </c>
+      <c r="D1109" t="inlineStr">
+        <is>
+          <t>command_success 检查禁用时不生成命令检查</t>
+        </is>
+      </c>
+    </row>
+    <row r="1110">
+      <c r="A1110" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1110" t="inlineStr">
+        <is>
+          <t>TestCommandSuccessCheck:</t>
+        </is>
+      </c>
+      <c r="C1110" t="inlineStr">
+        <is>
+          <t>test_multiple_nonzero_exit_codes</t>
+        </is>
+      </c>
+      <c r="D1110" t="inlineStr">
+        <is>
+          <t>多个非零退出码均被报告</t>
+        </is>
+      </c>
+    </row>
+    <row r="1111">
+      <c r="A1111" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1111" t="inlineStr">
+        <is>
+          <t>TestOnFailActions:</t>
+        </is>
+      </c>
+      <c r="C1111" t="inlineStr">
+        <is>
+          <t>test_annotate_appends_note</t>
+        </is>
+      </c>
+      <c r="D1111" t="inlineStr">
+        <is>
+          <t>on_fail=annotate 追加验证备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="1112">
+      <c r="A1112" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1112" t="inlineStr">
+        <is>
+          <t>TestOnFailActions:</t>
+        </is>
+      </c>
+      <c r="C1112" t="inlineStr">
+        <is>
+          <t>test_warn_appends_warning</t>
+        </is>
+      </c>
+      <c r="D1112" t="inlineStr">
+        <is>
+          <t>on_fail=warn 追加验证警告</t>
+        </is>
+      </c>
+    </row>
+    <row r="1113">
+      <c r="A1113" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1113" t="inlineStr">
+        <is>
+          <t>TestOnFailActions:</t>
+        </is>
+      </c>
+      <c r="C1113" t="inlineStr">
+        <is>
+          <t>test_block_with_high_severity</t>
+        </is>
+      </c>
+      <c r="D1113" t="inlineStr">
+        <is>
+          <t>on_fail=block 高严重度失败时阻塞输出</t>
+        </is>
+      </c>
+    </row>
+    <row r="1114">
+      <c r="A1114" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1114" t="inlineStr">
+        <is>
+          <t>TestOnFailActions:</t>
+        </is>
+      </c>
+      <c r="C1114" t="inlineStr">
+        <is>
+          <t>test_block_without_high_severity_does_not_block</t>
+        </is>
+      </c>
+      <c r="D1114" t="inlineStr">
+        <is>
+          <t>on_fail=block 无高严重度失败时不阻塞</t>
+        </is>
+      </c>
+    </row>
+    <row r="1115">
+      <c r="A1115" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1115" t="inlineStr">
+        <is>
+          <t>TestOnFailActions:</t>
+        </is>
+      </c>
+      <c r="C1115" t="inlineStr">
+        <is>
+          <t>test_annotate_is_default</t>
+        </is>
+      </c>
+      <c r="D1115" t="inlineStr">
+        <is>
+          <t>默认 on_fail 动作为 annotate</t>
+        </is>
+      </c>
+    </row>
+    <row r="1116">
+      <c r="A1116" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1116" t="inlineStr">
+        <is>
+          <t>TestOnPassActions:</t>
+        </is>
+      </c>
+      <c r="C1116" t="inlineStr">
+        <is>
+          <t>test_silent_is_default</t>
+        </is>
+      </c>
+      <c r="D1116" t="inlineStr">
+        <is>
+          <t>默认 on_pass 动作为 silent</t>
+        </is>
+      </c>
+    </row>
+    <row r="1117">
+      <c r="A1117" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1117" t="inlineStr">
+        <is>
+          <t>TestOnPassActions:</t>
+        </is>
+      </c>
+      <c r="C1117" t="inlineStr">
+        <is>
+          <t>test_silent_no_annotation</t>
+        </is>
+      </c>
+      <c r="D1117" t="inlineStr">
+        <is>
+          <t>on_pass=silent 全部通过时不修改响应</t>
+        </is>
+      </c>
+    </row>
+    <row r="1118">
+      <c r="A1118" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1118" t="inlineStr">
+        <is>
+          <t>TestOnPassActions:</t>
+        </is>
+      </c>
+      <c r="C1118" t="inlineStr">
+        <is>
+          <t>test_annotate_appends_pass_note</t>
+        </is>
+      </c>
+      <c r="D1118" t="inlineStr">
+        <is>
+          <t>on_pass=annotate 追加通过验证备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="1119">
+      <c r="A1119" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1119" t="inlineStr">
+        <is>
+          <t>TestNoChecksScenario:</t>
+        </is>
+      </c>
+      <c r="C1119" t="inlineStr">
+        <is>
+          <t>test_no_claims_no_checks</t>
+        </is>
+      </c>
+      <c r="D1119" t="inlineStr">
+        <is>
+          <t>无可验证声明时不生成检查</t>
+        </is>
+      </c>
+    </row>
+    <row r="1120">
+      <c r="A1120" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1120" t="inlineStr">
+        <is>
+          <t>TestNoChecksScenario:</t>
+        </is>
+      </c>
+      <c r="C1120" t="inlineStr">
+        <is>
+          <t>test_all_checks_pass_no_failure</t>
+        </is>
+      </c>
+      <c r="D1120" t="inlineStr">
+        <is>
+          <t>全部检查通过时 failed_checks 为空</t>
+        </is>
+      </c>
+    </row>
+    <row r="1121">
+      <c r="A1121" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1121" t="inlineStr">
+        <is>
+          <t>TestCustomValidators:</t>
+        </is>
+      </c>
+      <c r="C1121" t="inlineStr">
+        <is>
+          <t>test_custom_validator_pass</t>
+        </is>
+      </c>
+      <c r="D1121" t="inlineStr">
+        <is>
+          <t>自定义验证器通过时添加通过检查</t>
+        </is>
+      </c>
+    </row>
+    <row r="1122">
+      <c r="A1122" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1122" t="inlineStr">
+        <is>
+          <t>TestCustomValidators:</t>
+        </is>
+      </c>
+      <c r="C1122" t="inlineStr">
+        <is>
+          <t>test_custom_validator_fail</t>
+        </is>
+      </c>
+      <c r="D1122" t="inlineStr">
+        <is>
+          <t>自定义验证器失败时添加失败检查</t>
+        </is>
+      </c>
+    </row>
+    <row r="1123">
+      <c r="A1123" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1123" t="inlineStr">
+        <is>
+          <t>TestCustomValidators:</t>
+        </is>
+      </c>
+      <c r="C1123" t="inlineStr">
+        <is>
+          <t>test_custom_validator_exception_handled</t>
+        </is>
+      </c>
+      <c r="D1123" t="inlineStr">
+        <is>
+          <t>自定义验证器异常不影响验证流程</t>
+        </is>
+      </c>
+    </row>
+    <row r="1124">
+      <c r="A1124" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1124" t="inlineStr">
+        <is>
+          <t>TestCustomValidators:</t>
+        </is>
+      </c>
+      <c r="C1124" t="inlineStr">
+        <is>
+          <t>test_custom_validator_returns_none_skipped</t>
+        </is>
+      </c>
+      <c r="D1124" t="inlineStr">
+        <is>
+          <t>自定义验证器返回 None 时跳过</t>
+        </is>
+      </c>
+    </row>
+    <row r="1125">
+      <c r="A1125" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1125" t="inlineStr">
+        <is>
+          <t>TestEventEmission:</t>
+        </is>
+      </c>
+      <c r="C1125" t="inlineStr">
+        <is>
+          <t>test_blocked_emits_validation_failed_event</t>
+        </is>
+      </c>
+      <c r="D1125" t="inlineStr">
+        <is>
+          <t>阻塞时发出 VALIDATION_FAILED 事件</t>
+        </is>
+      </c>
+    </row>
+    <row r="1126">
+      <c r="A1126" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1126" t="inlineStr">
+        <is>
+          <t>TestEventEmission:</t>
+        </is>
+      </c>
+      <c r="C1126" t="inlineStr">
+        <is>
+          <t>test_blocked_emits_output_blocked_event</t>
+        </is>
+      </c>
+      <c r="D1126" t="inlineStr">
+        <is>
+          <t>阻塞时发出 OUTPUT_BLOCKED 事件</t>
+        </is>
+      </c>
+    </row>
+    <row r="1127">
+      <c r="A1127" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1127" t="inlineStr">
+        <is>
+          <t>TestEventEmission:</t>
+        </is>
+      </c>
+      <c r="C1127" t="inlineStr">
+        <is>
+          <t>test_no_events_when_not_blocked</t>
+        </is>
+      </c>
+      <c r="D1127" t="inlineStr">
+        <is>
+          <t>不阻塞时不发出 OUTPUT_BLOCKED 事件</t>
+        </is>
+      </c>
+    </row>
+    <row r="1128">
+      <c r="A1128" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1128" t="inlineStr">
+        <is>
+          <t>TestOrchestratorIntegration:</t>
+        </is>
+      </c>
+      <c r="C1128" t="inlineStr">
+        <is>
+          <t>test_validator_result_stored</t>
+        </is>
+      </c>
+      <c r="D1128" t="inlineStr">
+        <is>
+          <t>验证器结果存储为 last_validator_result</t>
+        </is>
+      </c>
+    </row>
+    <row r="1129">
+      <c r="A1129" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1129" t="inlineStr">
+        <is>
+          <t>TestOrchestratorIntegration:</t>
+        </is>
+      </c>
+      <c r="C1129" t="inlineStr">
+        <is>
+          <t>test_validator_not_set_when_none</t>
+        </is>
+      </c>
+      <c r="D1129" t="inlineStr">
+        <is>
+          <t>验证器为 None 时 last_validator_result 保持 None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1130">
+      <c r="A1130" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1130" t="inlineStr">
+        <is>
+          <t>TestPatternEdgeCases:</t>
+        </is>
+      </c>
+      <c r="C1130" t="inlineStr">
+        <is>
+          <t>test_short_path_ignored</t>
+        </is>
+      </c>
+      <c r="D1130" t="inlineStr">
+        <is>
+          <t>短路径被忽略不生成文件检查</t>
+        </is>
+      </c>
+    </row>
+    <row r="1131">
+      <c r="A1131" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1131" t="inlineStr">
+        <is>
+          <t>TestPatternEdgeCases:</t>
+        </is>
+      </c>
+      <c r="C1131" t="inlineStr">
+        <is>
+          <t>test_data_url_ignored</t>
+        </is>
+      </c>
+      <c r="D1131" t="inlineStr">
+        <is>
+          <t>data: URL 不被当作文件路径</t>
+        </is>
+      </c>
+    </row>
+    <row r="1132">
+      <c r="A1132" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1132" t="inlineStr">
+        <is>
+          <t>TestPatternEdgeCases:</t>
+        </is>
+      </c>
+      <c r="C1132" t="inlineStr">
+        <is>
+          <t>test_chinese_file_claim</t>
+        </is>
+      </c>
+      <c r="D1132" t="inlineStr">
+        <is>
+          <t>中文文件声明可正常检测</t>
+        </is>
+      </c>
+    </row>
+    <row r="1133">
+      <c r="A1133" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1133" t="inlineStr">
+        <is>
+          <t>TestPatternEdgeCases:</t>
+        </is>
+      </c>
+      <c r="C1133" t="inlineStr">
+        <is>
+          <t>test_code_claim_with_function</t>
+        </is>
+      </c>
+      <c r="D1133" t="inlineStr">
+        <is>
+          <t>含 function 关键词的代码正确性声明可检测</t>
+        </is>
+      </c>
+    </row>
+    <row r="1134">
+      <c r="A1134" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1134" t="inlineStr">
+        <is>
+          <t>TestPatternEdgeCases:</t>
+        </is>
+      </c>
+      <c r="C1134" t="inlineStr">
+        <is>
+          <t>test_command_claim_with_execution</t>
+        </is>
+      </c>
+      <c r="D1134" t="inlineStr">
+        <is>
+          <t>命令执行声明可被检测</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: v0.8.8 Schema-based 校验 — StandardToolOutput.data 格式 schema 验证 + 回退原始输出
- 新增 StandardToolOutput.validate(): 按 FORMAT_SCHEMAS 校验 required_keys + key_types
- 新增 FormatSchema frozen dataclass: 替代 stringly-typed plain dict 定义格式 schema
- 新增 _is_type_compatible(): 处理 bool ⊂ int 继承 + int → float 宽化
- 新增 ResultValidator.validate_tool_output(): 供 _observe() 调用，验证通过正常渲染，失败回退 result.output
- 新增 _emit_schema_failure(): schema 失败时发射 VALIDATION_FAILED 事件
- _observe() 集成: schema 验证在 to_llm_message() 前执行，失败时带可见标注前缀降级
- AgentSubsystems 门面: 新增 result_validator 参数，builder 通过门面注入
- ResultValidatorConfig.checks 默认列表添加 "schema"
- 5 种格式 schema: STATUS(必需status)/LIST(必需items+total)/CONTENT(必需source+content)/STRUCTURE(总通过)/ERROR(总通过)
- 29 个新测试: TestSchemaValidation(20) + TestIsTypeCompatible(7) + TestFormatSchema(2)
- 文档: api.md/architecture.md/constraints.md/tutorial.md 补全 schema 检查说明
- 全量 1650 测试通过

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/test_cases.xlsx
+++ b/tests/test_cases.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1134"/>
+  <dimension ref="A1:E1162"/>
   <sheetFormatPr baseColWidth="15" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27991,6 +27991,622 @@
         </is>
       </c>
     </row>
+    <row r="1135">
+      <c r="A1135" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1135" t="inlineStr">
+        <is>
+          <t>TestSchemaValidation:</t>
+        </is>
+      </c>
+      <c r="C1135" t="inlineStr">
+        <is>
+          <t>test_valid_status_schema_passes</t>
+        </is>
+      </c>
+      <c r="D1135" t="inlineStr">
+        <is>
+          <t>STATUS 格式完整数据通过 schema 验证</t>
+        </is>
+      </c>
+    </row>
+    <row r="1136">
+      <c r="A1136" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1136" t="inlineStr">
+        <is>
+          <t>TestSchemaValidation:</t>
+        </is>
+      </c>
+      <c r="C1136" t="inlineStr">
+        <is>
+          <t>test_status_missing_required_key</t>
+        </is>
+      </c>
+      <c r="D1136" t="inlineStr">
+        <is>
+          <t>STATUS 缺少 status 必需键被检测</t>
+        </is>
+      </c>
+    </row>
+    <row r="1137">
+      <c r="A1137" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1137" t="inlineStr">
+        <is>
+          <t>TestSchemaValidation:</t>
+        </is>
+      </c>
+      <c r="C1137" t="inlineStr">
+        <is>
+          <t>test_status_wrong_type</t>
+        </is>
+      </c>
+      <c r="D1137" t="inlineStr">
+        <is>
+          <t>STATUS exit_code 类型错误被检测</t>
+        </is>
+      </c>
+    </row>
+    <row r="1138">
+      <c r="A1138" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1138" t="inlineStr">
+        <is>
+          <t>TestSchemaValidation:</t>
+        </is>
+      </c>
+      <c r="C1138" t="inlineStr">
+        <is>
+          <t>test_status_python_executor_variant</t>
+        </is>
+      </c>
+      <c r="D1138" t="inlineStr">
+        <is>
+          <t>STATUS 使用 output 键（PythonExecutor 变体）通过验证</t>
+        </is>
+      </c>
+    </row>
+    <row r="1139">
+      <c r="A1139" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1139" t="inlineStr">
+        <is>
+          <t>TestSchemaValidation:</t>
+        </is>
+      </c>
+      <c r="C1139" t="inlineStr">
+        <is>
+          <t>test_list_schema_valid</t>
+        </is>
+      </c>
+      <c r="D1139" t="inlineStr">
+        <is>
+          <t>LIST 格式完整数据通过 schema 验证</t>
+        </is>
+      </c>
+    </row>
+    <row r="1140">
+      <c r="A1140" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1140" t="inlineStr">
+        <is>
+          <t>TestSchemaValidation:</t>
+        </is>
+      </c>
+      <c r="C1140" t="inlineStr">
+        <is>
+          <t>test_list_missing_items</t>
+        </is>
+      </c>
+      <c r="D1140" t="inlineStr">
+        <is>
+          <t>LIST 缺少 items 必需键被检测</t>
+        </is>
+      </c>
+    </row>
+    <row r="1141">
+      <c r="A1141" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1141" t="inlineStr">
+        <is>
+          <t>TestSchemaValidation:</t>
+        </is>
+      </c>
+      <c r="C1141" t="inlineStr">
+        <is>
+          <t>test_list_wrong_type_total</t>
+        </is>
+      </c>
+      <c r="D1141" t="inlineStr">
+        <is>
+          <t>LIST total 类型错误被检测</t>
+        </is>
+      </c>
+    </row>
+    <row r="1142">
+      <c r="A1142" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1142" t="inlineStr">
+        <is>
+          <t>TestSchemaValidation:</t>
+        </is>
+      </c>
+      <c r="C1142" t="inlineStr">
+        <is>
+          <t>test_content_schema_valid</t>
+        </is>
+      </c>
+      <c r="D1142" t="inlineStr">
+        <is>
+          <t>CONTENT 格式完整数据通过 schema 验证</t>
+        </is>
+      </c>
+    </row>
+    <row r="1143">
+      <c r="A1143" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1143" t="inlineStr">
+        <is>
+          <t>TestSchemaValidation:</t>
+        </is>
+      </c>
+      <c r="C1143" t="inlineStr">
+        <is>
+          <t>test_content_missing_source</t>
+        </is>
+      </c>
+      <c r="D1143" t="inlineStr">
+        <is>
+          <t>CONTENT 缺少 source 必需键被检测</t>
+        </is>
+      </c>
+    </row>
+    <row r="1144">
+      <c r="A1144" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1144" t="inlineStr">
+        <is>
+          <t>TestSchemaValidation:</t>
+        </is>
+      </c>
+      <c r="C1144" t="inlineStr">
+        <is>
+          <t>test_content_missing_content</t>
+        </is>
+      </c>
+      <c r="D1144" t="inlineStr">
+        <is>
+          <t>CONTENT 缺少 content 必需键被检测</t>
+        </is>
+      </c>
+    </row>
+    <row r="1145">
+      <c r="A1145" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1145" t="inlineStr">
+        <is>
+          <t>TestSchemaValidation:</t>
+        </is>
+      </c>
+      <c r="C1145" t="inlineStr">
+        <is>
+          <t>test_structure_always_passes</t>
+        </is>
+      </c>
+      <c r="D1145" t="inlineStr">
+        <is>
+          <t>STRUCTURE 格式总是通过验证</t>
+        </is>
+      </c>
+    </row>
+    <row r="1146">
+      <c r="A1146" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1146" t="inlineStr">
+        <is>
+          <t>TestSchemaValidation:</t>
+        </is>
+      </c>
+      <c r="C1146" t="inlineStr">
+        <is>
+          <t>test_error_schema_always_passes</t>
+        </is>
+      </c>
+      <c r="D1146" t="inlineStr">
+        <is>
+          <t>ERROR 格式含可选键时通过验证</t>
+        </is>
+      </c>
+    </row>
+    <row r="1147">
+      <c r="A1147" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1147" t="inlineStr">
+        <is>
+          <t>TestSchemaValidation:</t>
+        </is>
+      </c>
+      <c r="C1147" t="inlineStr">
+        <is>
+          <t>test_error_schema_empty_data_passes</t>
+        </is>
+      </c>
+      <c r="D1147" t="inlineStr">
+        <is>
+          <t>ERROR 格式空数据通过验证</t>
+        </is>
+      </c>
+    </row>
+    <row r="1148">
+      <c r="A1148" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1148" t="inlineStr">
+        <is>
+          <t>TestSchemaValidation:</t>
+        </is>
+      </c>
+      <c r="C1148" t="inlineStr">
+        <is>
+          <t>test_validate_tool_output_valid</t>
+        </is>
+      </c>
+      <c r="D1148" t="inlineStr">
+        <is>
+          <t>validate_tool_output() 有效输入返回 (True, [])</t>
+        </is>
+      </c>
+    </row>
+    <row r="1149">
+      <c r="A1149" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1149" t="inlineStr">
+        <is>
+          <t>TestSchemaValidation:</t>
+        </is>
+      </c>
+      <c r="C1149" t="inlineStr">
+        <is>
+          <t>test_validate_tool_output_invalid</t>
+        </is>
+      </c>
+      <c r="D1149" t="inlineStr">
+        <is>
+          <t>validate_tool_output() 无效输入返回 (False, errors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1150">
+      <c r="A1150" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1150" t="inlineStr">
+        <is>
+          <t>TestSchemaValidation:</t>
+        </is>
+      </c>
+      <c r="C1150" t="inlineStr">
+        <is>
+          <t>test_validate_tool_output_disabled_when_schema_not_in_checks</t>
+        </is>
+      </c>
+      <c r="D1150" t="inlineStr">
+        <is>
+          <t>schema 不在 checks 列表时 validate_tool_output() 跳过</t>
+        </is>
+      </c>
+    </row>
+    <row r="1151">
+      <c r="A1151" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1151" t="inlineStr">
+        <is>
+          <t>TestSchemaValidation:</t>
+        </is>
+      </c>
+      <c r="C1151" t="inlineStr">
+        <is>
+          <t>test_schema_check_not_in_validate_dispatch</t>
+        </is>
+      </c>
+      <c r="D1151" t="inlineStr">
+        <is>
+          <t>schema 不通过 validate() 文本路径分发</t>
+        </is>
+      </c>
+    </row>
+    <row r="1152">
+      <c r="A1152" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1152" t="inlineStr">
+        <is>
+          <t>TestSchemaValidation:</t>
+        </is>
+      </c>
+      <c r="C1152" t="inlineStr">
+        <is>
+          <t>test_validate_tool_output_emits_event</t>
+        </is>
+      </c>
+      <c r="D1152" t="inlineStr">
+        <is>
+          <t>schema 失败时发射 VALIDATION_FAILED 事件</t>
+        </is>
+      </c>
+    </row>
+    <row r="1153">
+      <c r="A1153" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1153" t="inlineStr">
+        <is>
+          <t>TestSchemaValidation:</t>
+        </is>
+      </c>
+      <c r="C1153" t="inlineStr">
+        <is>
+          <t>test_bool_value_rejected_for_int_key</t>
+        </is>
+      </c>
+      <c r="D1153" t="inlineStr">
+        <is>
+          <t>bool 值被 int 类型检查拒绝</t>
+        </is>
+      </c>
+    </row>
+    <row r="1154">
+      <c r="A1154" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1154" t="inlineStr">
+        <is>
+          <t>TestIsTypeCompatible:</t>
+        </is>
+      </c>
+      <c r="C1154" t="inlineStr">
+        <is>
+          <t>test_str_matches_str</t>
+        </is>
+      </c>
+      <c r="D1154" t="inlineStr">
+        <is>
+          <t>str 匹配 str 类型</t>
+        </is>
+      </c>
+    </row>
+    <row r="1155">
+      <c r="A1155" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1155" t="inlineStr">
+        <is>
+          <t>TestIsTypeCompatible:</t>
+        </is>
+      </c>
+      <c r="C1155" t="inlineStr">
+        <is>
+          <t>test_int_matches_int</t>
+        </is>
+      </c>
+      <c r="D1155" t="inlineStr">
+        <is>
+          <t>int 匹配 int 类型</t>
+        </is>
+      </c>
+    </row>
+    <row r="1156">
+      <c r="A1156" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1156" t="inlineStr">
+        <is>
+          <t>TestIsTypeCompatible:</t>
+        </is>
+      </c>
+      <c r="C1156" t="inlineStr">
+        <is>
+          <t>test_bool_rejected_for_int</t>
+        </is>
+      </c>
+      <c r="D1156" t="inlineStr">
+        <is>
+          <t>bool 被拒绝匹配 int 类型</t>
+        </is>
+      </c>
+    </row>
+    <row r="1157">
+      <c r="A1157" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1157" t="inlineStr">
+        <is>
+          <t>TestIsTypeCompatible:</t>
+        </is>
+      </c>
+      <c r="C1157" t="inlineStr">
+        <is>
+          <t>test_bool_accepted_for_bool</t>
+        </is>
+      </c>
+      <c r="D1157" t="inlineStr">
+        <is>
+          <t>bool 匹配 bool 类型</t>
+        </is>
+      </c>
+    </row>
+    <row r="1158">
+      <c r="A1158" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1158" t="inlineStr">
+        <is>
+          <t>TestIsTypeCompatible:</t>
+        </is>
+      </c>
+      <c r="C1158" t="inlineStr">
+        <is>
+          <t>test_int_accepted_for_float</t>
+        </is>
+      </c>
+      <c r="D1158" t="inlineStr">
+        <is>
+          <t>int 被接受匹配 float 类型</t>
+        </is>
+      </c>
+    </row>
+    <row r="1159">
+      <c r="A1159" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1159" t="inlineStr">
+        <is>
+          <t>TestIsTypeCompatible:</t>
+        </is>
+      </c>
+      <c r="C1159" t="inlineStr">
+        <is>
+          <t>test_str_rejected_for_int</t>
+        </is>
+      </c>
+      <c r="D1159" t="inlineStr">
+        <is>
+          <t>str 被拒绝匹配 int 类型</t>
+        </is>
+      </c>
+    </row>
+    <row r="1160">
+      <c r="A1160" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1160" t="inlineStr">
+        <is>
+          <t>TestIsTypeCompatible:</t>
+        </is>
+      </c>
+      <c r="C1160" t="inlineStr">
+        <is>
+          <t>test_list_matches_list</t>
+        </is>
+      </c>
+      <c r="D1160" t="inlineStr">
+        <is>
+          <t>list 匹配 list 类型</t>
+        </is>
+      </c>
+    </row>
+    <row r="1161">
+      <c r="A1161" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1161" t="inlineStr">
+        <is>
+          <t>TestFormatSchema:</t>
+        </is>
+      </c>
+      <c r="C1161" t="inlineStr">
+        <is>
+          <t>test_format_schemas_use_dataclass</t>
+        </is>
+      </c>
+      <c r="D1161" t="inlineStr">
+        <is>
+          <t>FORMAT_SCHEMAS 值均为 FormatSchema 实例</t>
+        </is>
+      </c>
+    </row>
+    <row r="1162">
+      <c r="A1162" t="inlineStr">
+        <is>
+          <t>result_validator</t>
+        </is>
+      </c>
+      <c r="B1162" t="inlineStr">
+        <is>
+          <t>TestFormatSchema:</t>
+        </is>
+      </c>
+      <c r="C1162" t="inlineStr">
+        <is>
+          <t>test_required_keys_are_tuple</t>
+        </is>
+      </c>
+      <c r="D1162" t="inlineStr">
+        <is>
+          <t>所有 schema 的 required_keys 为 tuple 类型</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: v0.9.0 流式执行 — Generator 事件流 + Ctrl+C 取消
run_stream() 作为核心实现返回 ExecutionHandle，run() 为 thin wrapper。
每阶段 yield ExecutionEvent（RUN_START/THINK/THINK_END/TOOL_CALL/
TOOL_RESULT/GUARD_SHORT_CIRCUIT/RUN_END/CANCELLED），CLI 实时显示
思考过程和工具调用，用户可 Ctrl+C 中断执行。

关键改动：
- types.py: ExecutionEventType 枚举 + ExecutionHandle(dataclass) +
  ExecutionEvent typed 字段 + TerminationReason.CANCELLED
- react.py: _think_stream() Generator 变体，run_stream() Generator
  实现，_guard_exit() 消除 5 处重复
- orchestrator.py: run_stream() 包装 agent generator + 后处理，
  抑制 agent 的 RUN_END 避免 double event
- main.py: 事件驱动 CLI 输出 + Ctrl+C 取消

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/test_cases.xlsx
+++ b/tests/test_cases.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1334"/>
+  <dimension ref="A1:E1350"/>
   <sheetFormatPr baseColWidth="15" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32391,6 +32391,358 @@
         </is>
       </c>
     </row>
+    <row r="1335">
+      <c r="A1335" t="inlineStr">
+        <is>
+          <t>streaming</t>
+        </is>
+      </c>
+      <c r="B1335" t="inlineStr">
+        <is>
+          <t>TestExecutionEventType</t>
+        </is>
+      </c>
+      <c r="C1335" t="inlineStr">
+        <is>
+          <t>test_all_event_types_defined</t>
+        </is>
+      </c>
+      <c r="D1335" t="inlineStr">
+        <is>
+          <t>ExecutionEventType 枚举包含全部 9 种事件类型</t>
+        </is>
+      </c>
+    </row>
+    <row r="1336">
+      <c r="A1336" t="inlineStr">
+        <is>
+          <t>streaming</t>
+        </is>
+      </c>
+      <c r="B1336" t="inlineStr">
+        <is>
+          <t>TestExecutionEventType</t>
+        </is>
+      </c>
+      <c r="C1336" t="inlineStr">
+        <is>
+          <t>test_event_type_values</t>
+        </is>
+      </c>
+      <c r="D1336" t="inlineStr">
+        <is>
+          <t>ExecutionEventType 枚举值与字符串匹配</t>
+        </is>
+      </c>
+    </row>
+    <row r="1337">
+      <c r="A1337" t="inlineStr">
+        <is>
+          <t>streaming</t>
+        </is>
+      </c>
+      <c r="B1337" t="inlineStr">
+        <is>
+          <t>TestExecutionEvent</t>
+        </is>
+      </c>
+      <c r="C1337" t="inlineStr">
+        <is>
+          <t>test_default_fields_are_none</t>
+        </is>
+      </c>
+      <c r="D1337" t="inlineStr">
+        <is>
+          <t>ExecutionEvent 默认 typed 字段为 None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1338">
+      <c r="A1338" t="inlineStr">
+        <is>
+          <t>streaming</t>
+        </is>
+      </c>
+      <c r="B1338" t="inlineStr">
+        <is>
+          <t>TestExecutionEvent</t>
+        </is>
+      </c>
+      <c r="C1338" t="inlineStr">
+        <is>
+          <t>test_typed_fields_populated</t>
+        </is>
+      </c>
+      <c r="D1338" t="inlineStr">
+        <is>
+          <t>ExecutionEvent typed 字段正确填充</t>
+        </is>
+      </c>
+    </row>
+    <row r="1339">
+      <c r="A1339" t="inlineStr">
+        <is>
+          <t>streaming</t>
+        </is>
+      </c>
+      <c r="B1339" t="inlineStr">
+        <is>
+          <t>TestExecutionHandle</t>
+        </is>
+      </c>
+      <c r="C1339" t="inlineStr">
+        <is>
+          <t>test_handle_wraps_generator</t>
+        </is>
+      </c>
+      <c r="D1339" t="inlineStr">
+        <is>
+          <t>ExecutionHandle 包装 generator 并可迭代</t>
+        </is>
+      </c>
+    </row>
+    <row r="1340">
+      <c r="A1340" t="inlineStr">
+        <is>
+          <t>streaming</t>
+        </is>
+      </c>
+      <c r="B1340" t="inlineStr">
+        <is>
+          <t>TestExecutionHandle</t>
+        </is>
+      </c>
+      <c r="C1340" t="inlineStr">
+        <is>
+          <t>test_cancel_sets_flag</t>
+        </is>
+      </c>
+      <c r="D1340" t="inlineStr">
+        <is>
+          <t>ExecutionHandle.cancel() 设置 cancelled 标志</t>
+        </is>
+      </c>
+    </row>
+    <row r="1341">
+      <c r="A1341" t="inlineStr">
+        <is>
+          <t>streaming</t>
+        </is>
+      </c>
+      <c r="B1341" t="inlineStr">
+        <is>
+          <t>TestThinkStream</t>
+        </is>
+      </c>
+      <c r="C1341" t="inlineStr">
+        <is>
+          <t>test_yields_think_events</t>
+        </is>
+      </c>
+      <c r="D1341" t="inlineStr">
+        <is>
+          <t>_think_stream() yield THINK_START/TEXT/END 并返回 ThinkResult</t>
+        </is>
+      </c>
+    </row>
+    <row r="1342">
+      <c r="A1342" t="inlineStr">
+        <is>
+          <t>streaming</t>
+        </is>
+      </c>
+      <c r="B1342" t="inlineStr">
+        <is>
+          <t>TestThinkStream</t>
+        </is>
+      </c>
+      <c r="C1342" t="inlineStr">
+        <is>
+          <t>test_think_wrapper_returns_same_result</t>
+        </is>
+      </c>
+      <c r="D1342" t="inlineStr">
+        <is>
+          <t>_think() 与 _think_stream() 返回相同 ThinkResult</t>
+        </is>
+      </c>
+    </row>
+    <row r="1343">
+      <c r="A1343" t="inlineStr">
+        <is>
+          <t>streaming</t>
+        </is>
+      </c>
+      <c r="B1343" t="inlineStr">
+        <is>
+          <t>TestRunStream</t>
+        </is>
+      </c>
+      <c r="C1343" t="inlineStr">
+        <is>
+          <t>test_simple_final_answer</t>
+        </is>
+      </c>
+      <c r="D1343" t="inlineStr">
+        <is>
+          <t>run_stream() 简单最终答案事件序列</t>
+        </is>
+      </c>
+    </row>
+    <row r="1344">
+      <c r="A1344" t="inlineStr">
+        <is>
+          <t>streaming</t>
+        </is>
+      </c>
+      <c r="B1344" t="inlineStr">
+        <is>
+          <t>TestRunStream</t>
+        </is>
+      </c>
+      <c r="C1344" t="inlineStr">
+        <is>
+          <t>test_one_tool_call_round</t>
+        </is>
+      </c>
+      <c r="D1344" t="inlineStr">
+        <is>
+          <t>run_stream() 一轮工具调用事件序列</t>
+        </is>
+      </c>
+    </row>
+    <row r="1345">
+      <c r="A1345" t="inlineStr">
+        <is>
+          <t>streaming</t>
+        </is>
+      </c>
+      <c r="B1345" t="inlineStr">
+        <is>
+          <t>TestRunStream</t>
+        </is>
+      </c>
+      <c r="C1345" t="inlineStr">
+        <is>
+          <t>test_guard_short_circuit</t>
+        </is>
+      </c>
+      <c r="D1345" t="inlineStr">
+        <is>
+          <t>run_stream() guard 短路 yield GUARD_SHORT_CIRCUIT + RUN_END</t>
+        </is>
+      </c>
+    </row>
+    <row r="1346">
+      <c r="A1346" t="inlineStr">
+        <is>
+          <t>streaming</t>
+        </is>
+      </c>
+      <c r="B1346" t="inlineStr">
+        <is>
+          <t>TestRunStream</t>
+        </is>
+      </c>
+      <c r="C1346" t="inlineStr">
+        <is>
+          <t>test_cancellation</t>
+        </is>
+      </c>
+      <c r="D1346" t="inlineStr">
+        <is>
+          <t>run_stream() 取消 yield CANCELLED + RUN_END</t>
+        </is>
+      </c>
+    </row>
+    <row r="1347">
+      <c r="A1347" t="inlineStr">
+        <is>
+          <t>streaming</t>
+        </is>
+      </c>
+      <c r="B1347" t="inlineStr">
+        <is>
+          <t>TestRunStream</t>
+        </is>
+      </c>
+      <c r="C1347" t="inlineStr">
+        <is>
+          <t>test_run_and_run_stream_equivalent</t>
+        </is>
+      </c>
+      <c r="D1347" t="inlineStr">
+        <is>
+          <t>run() 与 run_stream() 最终结果相同</t>
+        </is>
+      </c>
+    </row>
+    <row r="1348">
+      <c r="A1348" t="inlineStr">
+        <is>
+          <t>streaming</t>
+        </is>
+      </c>
+      <c r="B1348" t="inlineStr">
+        <is>
+          <t>TestOrchestratorRunStream</t>
+        </is>
+      </c>
+      <c r="C1348" t="inlineStr">
+        <is>
+          <t>test_basic_orchestrator_stream</t>
+        </is>
+      </c>
+      <c r="D1348" t="inlineStr">
+        <is>
+          <t>Orchestrator run_stream() 基本事件序列</t>
+        </is>
+      </c>
+    </row>
+    <row r="1349">
+      <c r="A1349" t="inlineStr">
+        <is>
+          <t>streaming</t>
+        </is>
+      </c>
+      <c r="B1349" t="inlineStr">
+        <is>
+          <t>TestOrchestratorRunStream</t>
+        </is>
+      </c>
+      <c r="C1349" t="inlineStr">
+        <is>
+          <t>test_run_and_run_stream_equivalent</t>
+        </is>
+      </c>
+      <c r="D1349" t="inlineStr">
+        <is>
+          <t>Orchestrator run() 与 run_stream() 结果等价</t>
+        </is>
+      </c>
+    </row>
+    <row r="1350">
+      <c r="A1350" t="inlineStr">
+        <is>
+          <t>streaming</t>
+        </is>
+      </c>
+      <c r="B1350" t="inlineStr">
+        <is>
+          <t>TestOrchestratorRunStream</t>
+        </is>
+      </c>
+      <c r="C1350" t="inlineStr">
+        <is>
+          <t>test_sanitizer_rejection_yields_run_end</t>
+        </is>
+      </c>
+      <c r="D1350" t="inlineStr">
+        <is>
+          <t>Sanitizer 拒绝 yield RUN_END + INPUT_REJECTED</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: v0.9.1 异步流式执行 — AsyncGenerator 逐 token 输出 + StreamingConfig
- LLM 层: StreamChunk 类型 + BaseLLM.chat_stream_async() 抽象接口
- 三个 Provider 异步流式实现 (Ollama/OpenAI/Anthropic)
- Agent 层: AsyncExecutionHandle + _think_stream_async() 逐 token THINK_TEXT
- 编排层: run_stream_async() + 取消传播
- CLI: run_interactive_async() + _handle_slash_command() 共享 23 个斜杠命令
- 配置: StreamingConfig(mode="sync"|"async") 默认同步向后兼容
- 文档: api.md/constraints.md/architecture.md/tutorial.md 同步更新
- 测试: 23 个异步流式测试 + 1824 全量测试通过

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/test_cases.xlsx
+++ b/tests/test_cases.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1350"/>
+  <dimension ref="A1:E1373"/>
   <sheetFormatPr baseColWidth="15" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32743,6 +32743,512 @@
         </is>
       </c>
     </row>
+    <row r="1351">
+      <c r="A1351" t="inlineStr">
+        <is>
+          <t>async_streaming</t>
+        </is>
+      </c>
+      <c r="B1351" t="inlineStr">
+        <is>
+          <t>TestStreamChunk</t>
+        </is>
+      </c>
+      <c r="C1351" t="inlineStr">
+        <is>
+          <t>test_default_values</t>
+        </is>
+      </c>
+      <c r="D1351" t="inlineStr">
+        <is>
+          <t>StreamChunk 默认值验证</t>
+        </is>
+      </c>
+    </row>
+    <row r="1352">
+      <c r="A1352" t="inlineStr">
+        <is>
+          <t>async_streaming</t>
+        </is>
+      </c>
+      <c r="B1352" t="inlineStr">
+        <is>
+          <t>TestStreamChunk</t>
+        </is>
+      </c>
+      <c r="C1352" t="inlineStr">
+        <is>
+          <t>test_text_chunk</t>
+        </is>
+      </c>
+      <c r="D1352" t="inlineStr">
+        <is>
+          <t>StreamChunk 文本块</t>
+        </is>
+      </c>
+    </row>
+    <row r="1353">
+      <c r="A1353" t="inlineStr">
+        <is>
+          <t>async_streaming</t>
+        </is>
+      </c>
+      <c r="B1353" t="inlineStr">
+        <is>
+          <t>TestStreamChunk</t>
+        </is>
+      </c>
+      <c r="C1353" t="inlineStr">
+        <is>
+          <t>test_tool_call_chunk</t>
+        </is>
+      </c>
+      <c r="D1353" t="inlineStr">
+        <is>
+          <t>StreamChunk 工具调用块</t>
+        </is>
+      </c>
+    </row>
+    <row r="1354">
+      <c r="A1354" t="inlineStr">
+        <is>
+          <t>async_streaming</t>
+        </is>
+      </c>
+      <c r="B1354" t="inlineStr">
+        <is>
+          <t>TestStreamChunk</t>
+        </is>
+      </c>
+      <c r="C1354" t="inlineStr">
+        <is>
+          <t>test_usage_chunk</t>
+        </is>
+      </c>
+      <c r="D1354" t="inlineStr">
+        <is>
+          <t>StreamChunk 用量块</t>
+        </is>
+      </c>
+    </row>
+    <row r="1355">
+      <c r="A1355" t="inlineStr">
+        <is>
+          <t>async_streaming</t>
+        </is>
+      </c>
+      <c r="B1355" t="inlineStr">
+        <is>
+          <t>TestAsyncExecutionHandle</t>
+        </is>
+      </c>
+      <c r="C1355" t="inlineStr">
+        <is>
+          <t>test_collect_result</t>
+        </is>
+      </c>
+      <c r="D1355" t="inlineStr">
+        <is>
+          <t>AsyncExecutionHandle 收集结果</t>
+        </is>
+      </c>
+    </row>
+    <row r="1356">
+      <c r="A1356" t="inlineStr">
+        <is>
+          <t>async_streaming</t>
+        </is>
+      </c>
+      <c r="B1356" t="inlineStr">
+        <is>
+          <t>TestAsyncExecutionHandle</t>
+        </is>
+      </c>
+      <c r="C1356" t="inlineStr">
+        <is>
+          <t>test_cancel</t>
+        </is>
+      </c>
+      <c r="D1356" t="inlineStr">
+        <is>
+          <t>AsyncExecutionHandle 取消</t>
+        </is>
+      </c>
+    </row>
+    <row r="1357">
+      <c r="A1357" t="inlineStr">
+        <is>
+          <t>async_streaming</t>
+        </is>
+      </c>
+      <c r="B1357" t="inlineStr">
+        <is>
+          <t>TestAsyncExecutionHandle</t>
+        </is>
+      </c>
+      <c r="C1357" t="inlineStr">
+        <is>
+          <t>test_collect_result_no_run_end</t>
+        </is>
+      </c>
+      <c r="D1357" t="inlineStr">
+        <is>
+          <t>AsyncExecutionHandle 无 RUN_END 返回 None</t>
+        </is>
+      </c>
+    </row>
+    <row r="1358">
+      <c r="A1358" t="inlineStr">
+        <is>
+          <t>async_streaming</t>
+        </is>
+      </c>
+      <c r="B1358" t="inlineStr">
+        <is>
+          <t>TestBaseLLMAsyncInterface</t>
+        </is>
+      </c>
+      <c r="C1358" t="inlineStr">
+        <is>
+          <t>test_ollama_has_async_impl</t>
+        </is>
+      </c>
+      <c r="D1358" t="inlineStr">
+        <is>
+          <t>OllamaLLM 实现 _chat_stream_async_impl</t>
+        </is>
+      </c>
+    </row>
+    <row r="1359">
+      <c r="A1359" t="inlineStr">
+        <is>
+          <t>async_streaming</t>
+        </is>
+      </c>
+      <c r="B1359" t="inlineStr">
+        <is>
+          <t>TestBaseLLMAsyncInterface</t>
+        </is>
+      </c>
+      <c r="C1359" t="inlineStr">
+        <is>
+          <t>test_openai_compatible_has_async_impl</t>
+        </is>
+      </c>
+      <c r="D1359" t="inlineStr">
+        <is>
+          <t>OpenAICompatibleLLM 实现 _chat_stream_async_impl</t>
+        </is>
+      </c>
+    </row>
+    <row r="1360">
+      <c r="A1360" t="inlineStr">
+        <is>
+          <t>async_streaming</t>
+        </is>
+      </c>
+      <c r="B1360" t="inlineStr">
+        <is>
+          <t>TestBaseLLMAsyncInterface</t>
+        </is>
+      </c>
+      <c r="C1360" t="inlineStr">
+        <is>
+          <t>test_anthropic_has_async_impl</t>
+        </is>
+      </c>
+      <c r="D1360" t="inlineStr">
+        <is>
+          <t>AnthropicLLM 实现 _chat_stream_async_impl</t>
+        </is>
+      </c>
+    </row>
+    <row r="1361">
+      <c r="A1361" t="inlineStr">
+        <is>
+          <t>async_streaming</t>
+        </is>
+      </c>
+      <c r="B1361" t="inlineStr">
+        <is>
+          <t>TestOllamaLLMAsyncStream</t>
+        </is>
+      </c>
+      <c r="C1361" t="inlineStr">
+        <is>
+          <t>test_text_streaming</t>
+        </is>
+      </c>
+      <c r="D1361" t="inlineStr">
+        <is>
+          <t>OllamaLLM 异步文本流</t>
+        </is>
+      </c>
+    </row>
+    <row r="1362">
+      <c r="A1362" t="inlineStr">
+        <is>
+          <t>async_streaming</t>
+        </is>
+      </c>
+      <c r="B1362" t="inlineStr">
+        <is>
+          <t>TestOllamaLLMAsyncStream</t>
+        </is>
+      </c>
+      <c r="C1362" t="inlineStr">
+        <is>
+          <t>test_tool_call_streaming</t>
+        </is>
+      </c>
+      <c r="D1362" t="inlineStr">
+        <is>
+          <t>OllamaLLM 异步工具调用流</t>
+        </is>
+      </c>
+    </row>
+    <row r="1363">
+      <c r="A1363" t="inlineStr">
+        <is>
+          <t>async_streaming</t>
+        </is>
+      </c>
+      <c r="B1363" t="inlineStr">
+        <is>
+          <t>TestOpenAICompatibleLLMAsyncStream</t>
+        </is>
+      </c>
+      <c r="C1363" t="inlineStr">
+        <is>
+          <t>test_text_streaming</t>
+        </is>
+      </c>
+      <c r="D1363" t="inlineStr">
+        <is>
+          <t>OpenAICompatibleLLM 异步文本流</t>
+        </is>
+      </c>
+    </row>
+    <row r="1364">
+      <c r="A1364" t="inlineStr">
+        <is>
+          <t>async_streaming</t>
+        </is>
+      </c>
+      <c r="B1364" t="inlineStr">
+        <is>
+          <t>TestOpenAICompatibleLLMAsyncStream</t>
+        </is>
+      </c>
+      <c r="C1364" t="inlineStr">
+        <is>
+          <t>test_tool_call_incremental</t>
+        </is>
+      </c>
+      <c r="D1364" t="inlineStr">
+        <is>
+          <t>OpenAICompatibleLLM 增量工具调用缓冲</t>
+        </is>
+      </c>
+    </row>
+    <row r="1365">
+      <c r="A1365" t="inlineStr">
+        <is>
+          <t>async_streaming</t>
+        </is>
+      </c>
+      <c r="B1365" t="inlineStr">
+        <is>
+          <t>TestAnthropicLLMAsyncStream</t>
+        </is>
+      </c>
+      <c r="C1365" t="inlineStr">
+        <is>
+          <t>test_text_streaming</t>
+        </is>
+      </c>
+      <c r="D1365" t="inlineStr">
+        <is>
+          <t>AnthropicLLM 异步文本流</t>
+        </is>
+      </c>
+    </row>
+    <row r="1366">
+      <c r="A1366" t="inlineStr">
+        <is>
+          <t>async_streaming</t>
+        </is>
+      </c>
+      <c r="B1366" t="inlineStr">
+        <is>
+          <t>TestAnthropicLLMAsyncStream</t>
+        </is>
+      </c>
+      <c r="C1366" t="inlineStr">
+        <is>
+          <t>test_tool_call_streaming</t>
+        </is>
+      </c>
+      <c r="D1366" t="inlineStr">
+        <is>
+          <t>AnthropicLLM 异步工具调用流</t>
+        </is>
+      </c>
+    </row>
+    <row r="1367">
+      <c r="A1367" t="inlineStr">
+        <is>
+          <t>async_streaming</t>
+        </is>
+      </c>
+      <c r="B1367" t="inlineStr">
+        <is>
+          <t>TestThinkStreamAsync</t>
+        </is>
+      </c>
+      <c r="C1367" t="inlineStr">
+        <is>
+          <t>test_token_by_token_think_text</t>
+        </is>
+      </c>
+      <c r="D1367" t="inlineStr">
+        <is>
+          <t>逐 token THINK_TEXT 事件</t>
+        </is>
+      </c>
+    </row>
+    <row r="1368">
+      <c r="A1368" t="inlineStr">
+        <is>
+          <t>async_streaming</t>
+        </is>
+      </c>
+      <c r="B1368" t="inlineStr">
+        <is>
+          <t>TestRunStreamAsyncSimpleAnswer</t>
+        </is>
+      </c>
+      <c r="C1368" t="inlineStr">
+        <is>
+          <t>test_simple_answer</t>
+        </is>
+      </c>
+      <c r="D1368" t="inlineStr">
+        <is>
+          <t>异步流式简单答案</t>
+        </is>
+      </c>
+    </row>
+    <row r="1369">
+      <c r="A1369" t="inlineStr">
+        <is>
+          <t>async_streaming</t>
+        </is>
+      </c>
+      <c r="B1369" t="inlineStr">
+        <is>
+          <t>TestRunStreamAsyncCancellation</t>
+        </is>
+      </c>
+      <c r="C1369" t="inlineStr">
+        <is>
+          <t>test_cancel_during_execution</t>
+        </is>
+      </c>
+      <c r="D1369" t="inlineStr">
+        <is>
+          <t>异步流式取消</t>
+        </is>
+      </c>
+    </row>
+    <row r="1370">
+      <c r="A1370" t="inlineStr">
+        <is>
+          <t>async_streaming</t>
+        </is>
+      </c>
+      <c r="B1370" t="inlineStr">
+        <is>
+          <t>TestSyncAsyncParity</t>
+        </is>
+      </c>
+      <c r="C1370" t="inlineStr">
+        <is>
+          <t>test_same_final_result</t>
+        </is>
+      </c>
+      <c r="D1370" t="inlineStr">
+        <is>
+          <t>同步/异步路径结果等价</t>
+        </is>
+      </c>
+    </row>
+    <row r="1371">
+      <c r="A1371" t="inlineStr">
+        <is>
+          <t>async_streaming</t>
+        </is>
+      </c>
+      <c r="B1371" t="inlineStr">
+        <is>
+          <t>TestStreamingConfig</t>
+        </is>
+      </c>
+      <c r="C1371" t="inlineStr">
+        <is>
+          <t>test_default_mode</t>
+        </is>
+      </c>
+      <c r="D1371" t="inlineStr">
+        <is>
+          <t>StreamingConfig 默认 mode=sync</t>
+        </is>
+      </c>
+    </row>
+    <row r="1372">
+      <c r="A1372" t="inlineStr">
+        <is>
+          <t>async_streaming</t>
+        </is>
+      </c>
+      <c r="B1372" t="inlineStr">
+        <is>
+          <t>TestStreamingConfig</t>
+        </is>
+      </c>
+      <c r="C1372" t="inlineStr">
+        <is>
+          <t>test_async_mode</t>
+        </is>
+      </c>
+      <c r="D1372" t="inlineStr">
+        <is>
+          <t>StreamingConfig mode=async</t>
+        </is>
+      </c>
+    </row>
+    <row r="1373">
+      <c r="A1373" t="inlineStr">
+        <is>
+          <t>async_streaming</t>
+        </is>
+      </c>
+      <c r="B1373" t="inlineStr">
+        <is>
+          <t>TestStreamingConfig</t>
+        </is>
+      </c>
+      <c r="C1373" t="inlineStr">
+        <is>
+          <t>test_config_has_streaming</t>
+        </is>
+      </c>
+      <c r="D1373" t="inlineStr">
+        <is>
+          <t>Config 包含 streaming 字段</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
test: 补充 get_base_chars() 初始化回归测试
验证 MetricsTracker 在未调用 start_run() 时 get_base_chars()
也能正常返回零值字典，而不抛出 AttributeError。

覆盖路径: MetricsTracker() → get_base_chars() （即 /context 命令路径）

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/test_cases.xlsx
+++ b/tests/test_cases.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1373"/>
+  <dimension ref="A1:E1374"/>
   <sheetFormatPr baseColWidth="15" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -33249,6 +33249,33 @@
         </is>
       </c>
     </row>
+    <row r="1374">
+      <c r="A1374" t="inlineStr">
+        <is>
+          <t>Monitoring</t>
+        </is>
+      </c>
+      <c r="B1374" t="inlineStr">
+        <is>
+          <t>TestBaseRatioFirstRoundCorrection</t>
+        </is>
+      </c>
+      <c r="C1374" t="inlineStr">
+        <is>
+          <t>test_get_base_chars_before_start_run</t>
+        </is>
+      </c>
+      <c r="D1374" t="inlineStr">
+        <is>
+          <t>MetricsTracker 在未调用 start_run() 时 get_base_chars() 也能正常返回零值字典</t>
+        </is>
+      </c>
+      <c r="E1374" t="inlineStr">
+        <is>
+          <t>AttributeError（__init__ 遗漏属性初始化）</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: BUG-006 StallDetector 签名改用结构特征，修复 Jaccard 相似度恒为 0
将 _make_signature() 中的 MD5 结果哈希替换为成功/失败状态 + 结果
量级分桶（0/small/medium/large/huge），使 Jaccard 相似度落在 0~1
之间，similarity_threshold 恢复正常工作。

同步更新测试：旧测试验证的是 MD5 行为（不同内容=不相似），更新为
验证结构特征行为（同工具+同规模+同成功=应停滞）。

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/test_cases.xlsx
+++ b/tests/test_cases.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1376"/>
+  <dimension ref="A1:E1379"/>
   <sheetFormatPr baseColWidth="15" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -33330,6 +33330,87 @@
         </is>
       </c>
     </row>
+    <row r="1377">
+      <c r="A1377" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="B1377" t="inlineStr">
+        <is>
+          <t>TestStallDetectorSimilarity</t>
+        </is>
+      </c>
+      <c r="C1377" t="inlineStr">
+        <is>
+          <t>test_same_tool_same_size_stall</t>
+        </is>
+      </c>
+      <c r="D1377" t="inlineStr">
+        <is>
+          <t>同工具+同规模+同成功状态应判定停滞（BUG-006 核心修复）</t>
+        </is>
+      </c>
+      <c r="E1377" t="inlineStr">
+        <is>
+          <t>StallDetector 相似度恒为 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="1378">
+      <c r="A1378" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="B1378" t="inlineStr">
+        <is>
+          <t>TestStallDetectorSimilarity</t>
+        </is>
+      </c>
+      <c r="C1378" t="inlineStr">
+        <is>
+          <t>test_different_size_no_stall</t>
+        </is>
+      </c>
+      <c r="D1378" t="inlineStr">
+        <is>
+          <t>不同结果量级不应判定停滞</t>
+        </is>
+      </c>
+      <c r="E1378" t="inlineStr">
+        <is>
+          <t>StallDetector 误判</t>
+        </is>
+      </c>
+    </row>
+    <row r="1379">
+      <c r="A1379" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="B1379" t="inlineStr">
+        <is>
+          <t>TestStallDetectorSimilarity</t>
+        </is>
+      </c>
+      <c r="C1379" t="inlineStr">
+        <is>
+          <t>test_fail_vs_success_no_stall</t>
+        </is>
+      </c>
+      <c r="D1379" t="inlineStr">
+        <is>
+          <t>失败结果与成功结果不应判定停滞</t>
+        </is>
+      </c>
+      <c r="E1379" t="inlineStr">
+        <is>
+          <t>StallDetector 误判</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: async 路径确认 handler 注册到 agent.events
orchestrator.events 和 agent.events 是独立的 EventEmitter，事件不转发。
async 路径的确认 handler 之前注册在 orchestrator.events 上，工具执行时
确认事件发在 agent.events，导致 handler 收不到事件，工具永久阻塞。

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/test_cases.xlsx
+++ b/tests/test_cases.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1381"/>
+  <dimension ref="A1:E1382"/>
   <sheetFormatPr baseColWidth="15" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -33465,6 +33465,33 @@
         </is>
       </c>
     </row>
+    <row r="1382">
+      <c r="A1382" t="inlineStr">
+        <is>
+          <t>Agent</t>
+        </is>
+      </c>
+      <c r="B1382" t="inlineStr">
+        <is>
+          <t>TestAgentOrchestrator</t>
+        </is>
+      </c>
+      <c r="C1382" t="inlineStr">
+        <is>
+          <t>test_orchestrator_and_agent_events_are_separate</t>
+        </is>
+      </c>
+      <c r="D1382" t="inlineStr">
+        <is>
+          <t>验证 orchestrator.events 和 agent.events 是独立的 EventEmitter，事件不转发</t>
+        </is>
+      </c>
+      <c r="E1382" t="inlineStr">
+        <is>
+          <t>async 路径确认 handler 收不到事件导致工具永久阻塞</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
refactor: 提取 provider normalizer 解耦 provider 差异
</commit_message>
<xml_diff>
--- a/tests/test_cases.xlsx
+++ b/tests/test_cases.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1382"/>
+  <dimension ref="A1:E1387"/>
   <sheetFormatPr baseColWidth="15" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -33492,6 +33492,129 @@
         </is>
       </c>
     </row>
+    <row r="1383">
+      <c r="A1383" t="inlineStr">
+        <is>
+          <t>LLM</t>
+        </is>
+      </c>
+      <c r="B1383" t="inlineStr">
+        <is>
+          <t>TestMessageNormalizer</t>
+        </is>
+      </c>
+      <c r="C1383" t="inlineStr">
+        <is>
+          <t>test_openai_normalizer_noop</t>
+        </is>
+      </c>
+      <c r="D1383" t="inlineStr">
+        <is>
+          <t>OpenAI normalizer 不修改消息</t>
+        </is>
+      </c>
+      <c r="E1383" t="inlineStr"/>
+    </row>
+    <row r="1384">
+      <c r="A1384" t="inlineStr">
+        <is>
+          <t>LLM</t>
+        </is>
+      </c>
+      <c r="B1384" t="inlineStr">
+        <is>
+          <t>TestMessageNormalizer</t>
+        </is>
+      </c>
+      <c r="C1384" t="inlineStr">
+        <is>
+          <t>test_deepseek_normalizer_adds_reasoning_content</t>
+        </is>
+      </c>
+      <c r="D1384" t="inlineStr">
+        <is>
+          <t>DeepSeek normalizer 补全空 reasoning_content</t>
+        </is>
+      </c>
+      <c r="E1384" t="inlineStr">
+        <is>
+          <t>DeepSeek API 400 错误</t>
+        </is>
+      </c>
+    </row>
+    <row r="1385">
+      <c r="A1385" t="inlineStr">
+        <is>
+          <t>LLM</t>
+        </is>
+      </c>
+      <c r="B1385" t="inlineStr">
+        <is>
+          <t>TestMessageNormalizer</t>
+        </is>
+      </c>
+      <c r="C1385" t="inlineStr">
+        <is>
+          <t>test_deepseek_normalizer_skips_if_present</t>
+        </is>
+      </c>
+      <c r="D1385" t="inlineStr">
+        <is>
+          <t>已有的 reasoning_content 不被覆盖</t>
+        </is>
+      </c>
+      <c r="E1385" t="inlineStr"/>
+    </row>
+    <row r="1386">
+      <c r="A1386" t="inlineStr">
+        <is>
+          <t>LLM</t>
+        </is>
+      </c>
+      <c r="B1386" t="inlineStr">
+        <is>
+          <t>TestMessageNormalizer</t>
+        </is>
+      </c>
+      <c r="C1386" t="inlineStr">
+        <is>
+          <t>test_xfyun_normalizer_skips_empty_id</t>
+        </is>
+      </c>
+      <c r="D1386" t="inlineStr">
+        <is>
+          <t>讯飞空 id/name 不覆盖已有值</t>
+        </is>
+      </c>
+      <c r="E1386" t="inlineStr">
+        <is>
+          <t>讯飞 SSE delta 覆盖 tool_call name</t>
+        </is>
+      </c>
+    </row>
+    <row r="1387">
+      <c r="A1387" t="inlineStr">
+        <is>
+          <t>LLM</t>
+        </is>
+      </c>
+      <c r="B1387" t="inlineStr">
+        <is>
+          <t>TestMessageNormalizer</t>
+        </is>
+      </c>
+      <c r="C1387" t="inlineStr">
+        <is>
+          <t>test_select_normalizer_by_model</t>
+        </is>
+      </c>
+      <c r="D1387" t="inlineStr">
+        <is>
+          <t>模型名匹配到正确的 Normalizer</t>
+        </is>
+      </c>
+      <c r="E1387" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>